<commit_message>
Dashboard: 2026-09-13 14:01 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G96"/>
+  <dimension ref="A1:G97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -3998,6 +3998,43 @@
         </is>
       </c>
       <c r="G96" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>13/09/2026 10:59</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>6518</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -6047,7 +6084,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -11873,7 +11910,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -32943,7 +32980,7 @@
       </c>
       <c r="F553" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G553" t="inlineStr">
@@ -38601,7 +38638,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 12/09/2026 10:14 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 13/09/2026 10:59 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57489,7 +57526,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 12/09/2026 10:14 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
+          <t>Atualizado: 13/09/2026 10:59 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -66935,7 +66972,7 @@
         </is>
       </c>
       <c r="B725" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C725" t="n">
         <v>0</v>
@@ -66944,7 +66981,7 @@
     <row r="727">
       <c r="A727" t="inlineStr">
         <is>
-          <t>Atualizado: 12/09/2026 10:14 | Total dias: 724</t>
+          <t>Atualizado: 13/09/2026 10:59 | Total dias: 724</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-14 16:07 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G97"/>
+  <dimension ref="A1:G98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4035,6 +4035,43 @@
         </is>
       </c>
       <c r="G97" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>14/09/2026 13:05</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>6522</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -23840,7 +23877,7 @@
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G378" t="inlineStr">
@@ -36629,7 +36666,7 @@
       </c>
       <c r="F623" t="inlineStr">
         <is>
-          <t>231</t>
+          <t>232</t>
         </is>
       </c>
       <c r="G623" t="inlineStr">
@@ -38638,7 +38675,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 13/09/2026 10:59 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 14/09/2026 13:05 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57526,7 +57563,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 13/09/2026 10:59 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
+          <t>Atualizado: 14/09/2026 13:05 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -57541,7 +57578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C727"/>
+  <dimension ref="A1:C729"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -66978,10 +67015,36 @@
         <v>0</v>
       </c>
     </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B726" t="n">
+        <v>1</v>
+      </c>
+      <c r="C726" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="727">
       <c r="A727" t="inlineStr">
         <is>
-          <t>Atualizado: 13/09/2026 10:59 | Total dias: 724</t>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B727" t="n">
+        <v>3</v>
+      </c>
+      <c r="C727" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>Atualizado: 14/09/2026 13:05 | Total dias: 726</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-15 14:34 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G98"/>
+  <dimension ref="A1:G99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4072,6 +4072,43 @@
         </is>
       </c>
       <c r="G98" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>15/09/2026 11:32</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>6522</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -38675,7 +38712,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 14/09/2026 13:05 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 15/09/2026 11:32 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57563,7 +57600,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 14/09/2026 13:05 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
+          <t>Atualizado: 15/09/2026 11:32 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -67044,7 +67081,7 @@
     <row r="729">
       <c r="A729" t="inlineStr">
         <is>
-          <t>Atualizado: 14/09/2026 13:05 | Total dias: 726</t>
+          <t>Atualizado: 15/09/2026 11:32 | Total dias: 726</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-16 14:31 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G99"/>
+  <dimension ref="A1:G100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4109,6 +4109,43 @@
         </is>
       </c>
       <c r="G99" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>16/09/2026 11:29</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>6524</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -38712,7 +38749,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 15/09/2026 11:32 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 16/09/2026 11:29 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57600,7 +57637,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 15/09/2026 11:32 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
+          <t>Atualizado: 16/09/2026 11:29 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -57615,7 +57652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C729"/>
+  <dimension ref="A1:C730"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -67078,10 +67115,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="729">
-      <c r="A729" t="inlineStr">
-        <is>
-          <t>Atualizado: 15/09/2026 11:32 | Total dias: 726</t>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>15/09/2026</t>
+        </is>
+      </c>
+      <c r="B728" t="n">
+        <v>2</v>
+      </c>
+      <c r="C728" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>Atualizado: 16/09/2026 11:29 | Total dias: 727</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-17 14:35 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G100"/>
+  <dimension ref="A1:G101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4146,6 +4146,43 @@
         </is>
       </c>
       <c r="G100" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>17/09/2026 11:33</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>6531</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -7029,7 +7066,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -12860,7 +12897,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>97</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
@@ -23268,7 +23305,7 @@
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G365" t="inlineStr">
@@ -31260,7 +31297,7 @@
       </c>
       <c r="F518" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G518" t="inlineStr">
@@ -32624,7 +32661,7 @@
       </c>
       <c r="F544" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G544" t="inlineStr">
@@ -36740,7 +36777,7 @@
       </c>
       <c r="F623" t="inlineStr">
         <is>
-          <t>232</t>
+          <t>233</t>
         </is>
       </c>
       <c r="G623" t="inlineStr">
@@ -38749,7 +38786,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 16/09/2026 11:29 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 17/09/2026 11:33 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57637,7 +57674,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 16/09/2026 11:29 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
+          <t>Atualizado: 17/09/2026 11:33 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -57652,7 +57689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C730"/>
+  <dimension ref="A1:C732"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -67128,10 +67165,36 @@
         <v>0</v>
       </c>
     </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+      <c r="B729" t="n">
+        <v>6</v>
+      </c>
+      <c r="C729" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="730">
       <c r="A730" t="inlineStr">
         <is>
-          <t>Atualizado: 16/09/2026 11:29 | Total dias: 727</t>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B730" t="n">
+        <v>1</v>
+      </c>
+      <c r="C730" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>Atualizado: 17/09/2026 11:33 | Total dias: 729</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-18 14:00 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:G102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4183,6 +4183,43 @@
         </is>
       </c>
       <c r="G101" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>18/09/2026 10:58</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>6536</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -16454,7 +16491,7 @@
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G234" t="inlineStr">
@@ -35993,7 +36030,7 @@
       </c>
       <c r="F608" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>71</t>
         </is>
       </c>
       <c r="G608" t="inlineStr">
@@ -36777,7 +36814,7 @@
       </c>
       <c r="F623" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>235</t>
         </is>
       </c>
       <c r="G623" t="inlineStr">
@@ -38786,7 +38823,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 17/09/2026 11:33 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 18/09/2026 10:58 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57674,7 +57711,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 17/09/2026 11:33 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
+          <t>Atualizado: 18/09/2026 10:58 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -57689,7 +57726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C732"/>
+  <dimension ref="A1:C733"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -67185,16 +67222,29 @@
         </is>
       </c>
       <c r="B730" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C730" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="732">
-      <c r="A732" t="inlineStr">
-        <is>
-          <t>Atualizado: 17/09/2026 11:33 | Total dias: 729</t>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>18/09/2026</t>
+        </is>
+      </c>
+      <c r="B731" t="n">
+        <v>2</v>
+      </c>
+      <c r="C731" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>Atualizado: 18/09/2026 10:58 | Total dias: 730</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-19 13:37 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G102"/>
+  <dimension ref="A1:G103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4220,6 +4220,43 @@
         </is>
       </c>
       <c r="G102" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>19/09/2026 10:35</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>6540</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -38823,7 +38860,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 18/09/2026 10:58 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 19/09/2026 10:35 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57711,7 +57748,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 18/09/2026 10:58 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
+          <t>Atualizado: 19/09/2026 10:35 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -67235,7 +67272,7 @@
         </is>
       </c>
       <c r="B731" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C731" t="n">
         <v>0</v>
@@ -67244,7 +67281,7 @@
     <row r="733">
       <c r="A733" t="inlineStr">
         <is>
-          <t>Atualizado: 18/09/2026 10:58 | Total dias: 730</t>
+          <t>Atualizado: 19/09/2026 10:35 | Total dias: 730</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-20 13:50 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G103"/>
+  <dimension ref="A1:G104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4257,6 +4257,43 @@
         </is>
       </c>
       <c r="G103" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>20/09/2026 10:48</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>6542</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -6775,7 +6812,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -38860,7 +38897,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 19/09/2026 10:35 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 20/09/2026 10:48 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57748,7 +57785,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 19/09/2026 10:35 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
+          <t>Atualizado: 20/09/2026 10:48 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -57763,7 +57800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C733"/>
+  <dimension ref="A1:C734"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -67278,10 +67315,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="733">
-      <c r="A733" t="inlineStr">
-        <is>
-          <t>Atualizado: 19/09/2026 10:35 | Total dias: 730</t>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>19/09/2026</t>
+        </is>
+      </c>
+      <c r="B732" t="n">
+        <v>2</v>
+      </c>
+      <c r="C732" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>Atualizado: 20/09/2026 10:48 | Total dias: 731</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-21 16:09 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G104"/>
+  <dimension ref="A1:G105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4294,6 +4294,43 @@
         </is>
       </c>
       <c r="G104" t="inlineStr">
+        <is>
+          <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>21/09/2026 13:07</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>6546</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
         <is>
           <t>514</t>
         </is>
@@ -6238,7 +6275,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -13008,7 +13045,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>97</t>
+          <t>98</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
@@ -36888,7 +36925,7 @@
       </c>
       <c r="F623" t="inlineStr">
         <is>
-          <t>235</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G623" t="inlineStr">
@@ -38897,7 +38934,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 20/09/2026 10:48 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 21/09/2026 13:07 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -57785,7 +57822,7 @@
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 20/09/2026 10:48 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
+          <t>Atualizado: 21/09/2026 13:07 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
         </is>
       </c>
     </row>
@@ -57800,7 +57837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C734"/>
+  <dimension ref="A1:C736"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -67328,10 +67365,36 @@
         <v>0</v>
       </c>
     </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>20/09/2026</t>
+        </is>
+      </c>
+      <c r="B733" t="n">
+        <v>2</v>
+      </c>
+      <c r="C733" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="734">
       <c r="A734" t="inlineStr">
         <is>
-          <t>Atualizado: 20/09/2026 10:48 | Total dias: 731</t>
+          <t>21/09/2026</t>
+        </is>
+      </c>
+      <c r="B734" t="n">
+        <v>2</v>
+      </c>
+      <c r="C734" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>Atualizado: 21/09/2026 13:07 | Total dias: 733</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-22 14:19 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G105"/>
+  <dimension ref="A1:G106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4333,6 +4333,43 @@
       <c r="G105" t="inlineStr">
         <is>
           <t>514</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>22/09/2026 11:16</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>844</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>6552</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>707</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>516</t>
         </is>
       </c>
     </row>
@@ -6432,7 +6469,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -9052,7 +9089,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -9370,7 +9407,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -15395,7 +15432,7 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
@@ -24816,7 +24853,7 @@
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="G391" t="inlineStr">
@@ -35673,7 +35710,7 @@
       </c>
       <c r="F599" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G599" t="inlineStr">
@@ -38934,7 +38971,7 @@
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>Atualizado: 21/09/2026 13:07 | Ativas: 844 | Inativas: 0</t>
+          <t>Atualizado: 22/09/2026 11:16 | Ativas: 844 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -38949,7 +38986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E708"/>
+  <dimension ref="A1:E710"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -57819,10 +57856,64 @@
         </is>
       </c>
     </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>969</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>Colosso Fortaleza</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>Nao cadastrado</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>EVENTOS</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
     <row r="708">
       <c r="A708" t="inlineStr">
         <is>
-          <t>Atualizado: 21/09/2026 13:07 | Total: 705 | c/ usuario: 191 | s/ usuario: 514</t>
+          <t>970</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>ERS - English School for Women</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>Nao cadastrado</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>EDUCAÇÃO</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>Atualizado: 22/09/2026 11:16 | Total: 707 | c/ usuario: 191 | s/ usuario: 516</t>
         </is>
       </c>
     </row>
@@ -67385,7 +67476,7 @@
         </is>
       </c>
       <c r="B734" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C734" t="n">
         <v>0</v>
@@ -67394,7 +67485,7 @@
     <row r="736">
       <c r="A736" t="inlineStr">
         <is>
-          <t>Atualizado: 21/09/2026 13:07 | Total dias: 733</t>
+          <t>Atualizado: 22/09/2026 11:16 | Total dias: 733</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-26 13:59 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G109"/>
+  <dimension ref="A1:G110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4479,6 +4479,43 @@
         </is>
       </c>
       <c r="G109" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>26/09/2026 10:57</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>849</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>6578</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>711</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>196</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -19058,7 +19095,7 @@
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
@@ -39342,7 +39379,7 @@
     <row r="668">
       <c r="A668" t="inlineStr">
         <is>
-          <t>Atualizado: 25/09/2026 11:53 | Ativas: 849 | Inativas: 0</t>
+          <t>Atualizado: 26/09/2026 10:57 | Ativas: 849 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -58386,7 +58423,7 @@
     <row r="714">
       <c r="A714" t="inlineStr">
         <is>
-          <t>Atualizado: 25/09/2026 11:53 | Total: 711 | c/ usuario: 196 | s/ usuario: 515</t>
+          <t>Atualizado: 26/09/2026 10:57 | Total: 711 | c/ usuario: 196 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -58401,7 +58438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C740"/>
+  <dimension ref="A1:C741"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68001,16 +68038,29 @@
         </is>
       </c>
       <c r="B738" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C738" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="740">
-      <c r="A740" t="inlineStr">
-        <is>
-          <t>Atualizado: 25/09/2026 11:53 | Total dias: 737</t>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B739" t="n">
+        <v>2</v>
+      </c>
+      <c r="C739" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>Atualizado: 26/09/2026 10:57 | Total dias: 738</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-27 14:55 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G110"/>
+  <dimension ref="A1:G111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4516,6 +4516,43 @@
         </is>
       </c>
       <c r="G110" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>27/09/2026 11:53</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>849</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>6586</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>185</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>711</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>196</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -5153,7 +5190,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -13282,7 +13319,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>151</t>
+          <t>152</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -16421,7 +16458,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
@@ -39379,7 +39416,7 @@
     <row r="668">
       <c r="A668" t="inlineStr">
         <is>
-          <t>Atualizado: 26/09/2026 10:57 | Ativas: 849 | Inativas: 0</t>
+          <t>Atualizado: 27/09/2026 11:53 | Ativas: 849 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -58423,7 +58460,7 @@
     <row r="714">
       <c r="A714" t="inlineStr">
         <is>
-          <t>Atualizado: 26/09/2026 10:57 | Total: 711 | c/ usuario: 196 | s/ usuario: 515</t>
+          <t>Atualizado: 27/09/2026 11:53 | Total: 711 | c/ usuario: 196 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -58438,7 +58475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C741"/>
+  <dimension ref="A1:C742"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68051,16 +68088,29 @@
         </is>
       </c>
       <c r="B739" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C739" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="741">
-      <c r="A741" t="inlineStr">
-        <is>
-          <t>Atualizado: 26/09/2026 10:57 | Total dias: 738</t>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="B740" t="n">
+        <v>4</v>
+      </c>
+      <c r="C740" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>Atualizado: 27/09/2026 11:53 | Total dias: 739</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-28 17:55 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G111"/>
+  <dimension ref="A1:G112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4553,6 +4553,43 @@
         </is>
       </c>
       <c r="G111" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>28/09/2026 14:52</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>849</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>6592</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>185</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>711</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>196</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -25923,7 +25960,7 @@
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G408" t="inlineStr">
@@ -26289,7 +26326,7 @@
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="G415" t="inlineStr">
@@ -27386,7 +27423,7 @@
       </c>
       <c r="F436" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G436" t="inlineStr">
@@ -39416,7 +39453,7 @@
     <row r="668">
       <c r="A668" t="inlineStr">
         <is>
-          <t>Atualizado: 27/09/2026 11:53 | Ativas: 849 | Inativas: 0</t>
+          <t>Atualizado: 28/09/2026 14:52 | Ativas: 849 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -58460,7 +58497,7 @@
     <row r="714">
       <c r="A714" t="inlineStr">
         <is>
-          <t>Atualizado: 27/09/2026 11:53 | Total: 711 | c/ usuario: 196 | s/ usuario: 515</t>
+          <t>Atualizado: 28/09/2026 14:52 | Total: 711 | c/ usuario: 196 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -58475,7 +58512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C742"/>
+  <dimension ref="A1:C743"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68101,16 +68138,29 @@
         </is>
       </c>
       <c r="B740" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C740" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="742">
-      <c r="A742" t="inlineStr">
-        <is>
-          <t>Atualizado: 27/09/2026 11:53 | Total dias: 739</t>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="B741" t="n">
+        <v>1</v>
+      </c>
+      <c r="C741" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>Atualizado: 28/09/2026 14:52 | Total dias: 740</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-29 16:17 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G112"/>
+  <dimension ref="A1:G113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4590,6 +4590,43 @@
         </is>
       </c>
       <c r="G112" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>29/09/2026 13:15</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>849</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>6602</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>185</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>711</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>196</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -8151,7 +8188,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -13356,7 +13393,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>153</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -22617,7 +22654,7 @@
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
@@ -23920,7 +23957,7 @@
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G369" t="inlineStr">
@@ -26326,7 +26363,7 @@
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G415" t="inlineStr">
@@ -32434,7 +32471,7 @@
       </c>
       <c r="F532" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G532" t="inlineStr">
@@ -34367,7 +34404,7 @@
       </c>
       <c r="F569" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G569" t="inlineStr">
@@ -39453,7 +39490,7 @@
     <row r="668">
       <c r="A668" t="inlineStr">
         <is>
-          <t>Atualizado: 28/09/2026 14:52 | Ativas: 849 | Inativas: 0</t>
+          <t>Atualizado: 29/09/2026 13:15 | Ativas: 849 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -58497,7 +58534,7 @@
     <row r="714">
       <c r="A714" t="inlineStr">
         <is>
-          <t>Atualizado: 28/09/2026 14:52 | Total: 711 | c/ usuario: 196 | s/ usuario: 515</t>
+          <t>Atualizado: 29/09/2026 13:15 | Total: 711 | c/ usuario: 196 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -58512,7 +58549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C743"/>
+  <dimension ref="A1:C744"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68151,16 +68188,29 @@
         </is>
       </c>
       <c r="B741" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C741" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="743">
-      <c r="A743" t="inlineStr">
-        <is>
-          <t>Atualizado: 28/09/2026 14:52 | Total dias: 740</t>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="B742" t="n">
+        <v>4</v>
+      </c>
+      <c r="C742" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>Atualizado: 29/09/2026 13:15 | Total dias: 741</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-09-30 16:13 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G113"/>
+  <dimension ref="A1:G114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4627,6 +4627,43 @@
         </is>
       </c>
       <c r="G113" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>30/09/2026 13:10</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>849</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>6611</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>186</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>711</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>196</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -9719,7 +9756,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -15481,7 +15518,7 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
@@ -22811,7 +22848,7 @@
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
@@ -26363,7 +26400,7 @@
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="G415" t="inlineStr">
@@ -31896,7 +31933,7 @@
       </c>
       <c r="F521" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="G521" t="inlineStr">
@@ -36593,7 +36630,7 @@
       </c>
       <c r="F611" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G611" t="inlineStr">
@@ -39490,7 +39527,7 @@
     <row r="668">
       <c r="A668" t="inlineStr">
         <is>
-          <t>Atualizado: 29/09/2026 13:15 | Ativas: 849 | Inativas: 0</t>
+          <t>Atualizado: 30/09/2026 13:10 | Ativas: 849 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -58534,7 +58571,7 @@
     <row r="714">
       <c r="A714" t="inlineStr">
         <is>
-          <t>Atualizado: 29/09/2026 13:15 | Total: 711 | c/ usuario: 196 | s/ usuario: 515</t>
+          <t>Atualizado: 30/09/2026 13:10 | Total: 711 | c/ usuario: 196 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -58549,7 +58586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C744"/>
+  <dimension ref="A1:C745"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68201,16 +68238,29 @@
         </is>
       </c>
       <c r="B742" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C742" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="744">
-      <c r="A744" t="inlineStr">
-        <is>
-          <t>Atualizado: 29/09/2026 13:15 | Total dias: 741</t>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="B743" t="n">
+        <v>7</v>
+      </c>
+      <c r="C743" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>Atualizado: 30/09/2026 13:10 | Total dias: 742</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-01 16:57 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G114"/>
+  <dimension ref="A1:G115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4664,6 +4664,43 @@
         </is>
       </c>
       <c r="G114" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>01/10/2026 13:54</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>849</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>6617</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>186</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>711</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>196</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -14578,7 +14615,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
@@ -20337,7 +20374,7 @@
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>45</t>
         </is>
       </c>
       <c r="G299" t="inlineStr">
@@ -32876,7 +32913,7 @@
       </c>
       <c r="F539" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="G539" t="inlineStr">
@@ -36890,7 +36927,7 @@
       </c>
       <c r="F616" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="G616" t="inlineStr">
@@ -38615,7 +38652,7 @@
       </c>
       <c r="F649" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G649" t="inlineStr">
@@ -39527,7 +39564,7 @@
     <row r="668">
       <c r="A668" t="inlineStr">
         <is>
-          <t>Atualizado: 30/09/2026 13:10 | Ativas: 849 | Inativas: 0</t>
+          <t>Atualizado: 01/10/2026 13:54 | Ativas: 849 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -58571,7 +58608,7 @@
     <row r="714">
       <c r="A714" t="inlineStr">
         <is>
-          <t>Atualizado: 30/09/2026 13:10 | Total: 711 | c/ usuario: 196 | s/ usuario: 515</t>
+          <t>Atualizado: 01/10/2026 13:54 | Total: 711 | c/ usuario: 196 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -58586,7 +58623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C745"/>
+  <dimension ref="A1:C746"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68251,16 +68288,29 @@
         </is>
       </c>
       <c r="B743" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C743" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="745">
-      <c r="A745" t="inlineStr">
-        <is>
-          <t>Atualizado: 30/09/2026 13:10 | Total dias: 742</t>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B744" t="n">
+        <v>5</v>
+      </c>
+      <c r="C744" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>Atualizado: 01/10/2026 13:54 | Total dias: 743</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-02 16:04 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G115"/>
+  <dimension ref="A1:G116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4701,6 +4701,43 @@
         </is>
       </c>
       <c r="G115" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>02/10/2026 13:02</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>849</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>6622</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>187</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>711</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>196</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -9636,7 +9673,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -16398,12 +16435,12 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H223" t="inlineStr">
@@ -28656,17 +28693,17 @@
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>20% OFF</t>
         </is>
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>1622</t>
+          <t>1518</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D458" t="inlineStr">
@@ -28701,24 +28738,24 @@
       </c>
       <c r="J458" t="inlineStr">
         <is>
-          <t>969</t>
+          <t>884</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t>20% OFF</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>1518</t>
+          <t>1622</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D459" t="inlineStr">
@@ -28733,7 +28770,7 @@
       </c>
       <c r="F459" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G459" t="inlineStr">
@@ -28753,7 +28790,7 @@
       </c>
       <c r="J459" t="inlineStr">
         <is>
-          <t>884</t>
+          <t>969</t>
         </is>
       </c>
     </row>
@@ -29358,7 +29395,7 @@
       </c>
       <c r="F471" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="G471" t="inlineStr">
@@ -39564,7 +39601,7 @@
     <row r="668">
       <c r="A668" t="inlineStr">
         <is>
-          <t>Atualizado: 01/10/2026 13:54 | Ativas: 849 | Inativas: 0</t>
+          <t>Atualizado: 02/10/2026 13:02 | Ativas: 849 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -58608,7 +58645,7 @@
     <row r="714">
       <c r="A714" t="inlineStr">
         <is>
-          <t>Atualizado: 01/10/2026 13:54 | Total: 711 | c/ usuario: 196 | s/ usuario: 515</t>
+          <t>Atualizado: 02/10/2026 13:02 | Total: 711 | c/ usuario: 196 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -58623,7 +58660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C746"/>
+  <dimension ref="A1:C747"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68301,16 +68338,29 @@
         </is>
       </c>
       <c r="B744" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C744" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="B745" t="n">
+        <v>1</v>
+      </c>
+      <c r="C745" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="746">
-      <c r="A746" t="inlineStr">
-        <is>
-          <t>Atualizado: 01/10/2026 13:54 | Total dias: 743</t>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>Atualizado: 02/10/2026 13:02 | Total dias: 744</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-03 14:32 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G116"/>
+  <dimension ref="A1:G117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4738,6 +4738,43 @@
         </is>
       </c>
       <c r="G116" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>03/10/2026 11:29</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>6626</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>187</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -4754,7 +4791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J668"/>
+  <dimension ref="A1:J669"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -26474,7 +26511,7 @@
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="G415" t="inlineStr">
@@ -34750,17 +34787,17 @@
     <row r="574">
       <c r="A574" t="inlineStr">
         <is>
-          <t>SOBREMESA</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B574" t="inlineStr">
         <is>
-          <t>1396</t>
+          <t>1623</t>
         </is>
       </c>
       <c r="C574" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D574" t="inlineStr">
@@ -34775,7 +34812,7 @@
       </c>
       <c r="F574" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G574" t="inlineStr">
@@ -34795,24 +34832,24 @@
       </c>
       <c r="J574" t="inlineStr">
         <is>
-          <t>766</t>
+          <t>975</t>
         </is>
       </c>
     </row>
     <row r="575">
       <c r="A575" t="inlineStr">
         <is>
-          <t>5% OFF em Eventos</t>
+          <t>SOBREMESA</t>
         </is>
       </c>
       <c r="B575" t="inlineStr">
         <is>
-          <t>1534</t>
+          <t>1396</t>
         </is>
       </c>
       <c r="C575" t="inlineStr">
         <is>
-          <t>5.00%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D575" t="inlineStr">
@@ -34827,7 +34864,7 @@
       </c>
       <c r="F575" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G575" t="inlineStr">
@@ -34847,24 +34884,24 @@
       </c>
       <c r="J575" t="inlineStr">
         <is>
-          <t>898</t>
+          <t>766</t>
         </is>
       </c>
     </row>
     <row r="576">
       <c r="A576" t="inlineStr">
         <is>
-          <t>Frete grátis para os alunos da Greenlife</t>
+          <t>5% OFF em Eventos</t>
         </is>
       </c>
       <c r="B576" t="inlineStr">
         <is>
-          <t>1066</t>
+          <t>1534</t>
         </is>
       </c>
       <c r="C576" t="inlineStr">
         <is>
-          <t>R$ 0.00</t>
+          <t>5.00%</t>
         </is>
       </c>
       <c r="D576" t="inlineStr">
@@ -34879,7 +34916,7 @@
       </c>
       <c r="F576" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G576" t="inlineStr">
@@ -34899,19 +34936,19 @@
       </c>
       <c r="J576" t="inlineStr">
         <is>
-          <t>428</t>
+          <t>898</t>
         </is>
       </c>
     </row>
     <row r="577">
       <c r="A577" t="inlineStr">
         <is>
-          <t>500 mb de R$ 109,90 por R$ 79,90 nos 2 primeiros meses.</t>
+          <t>Frete grátis para os alunos da Greenlife</t>
         </is>
       </c>
       <c r="B577" t="inlineStr">
         <is>
-          <t>973</t>
+          <t>1066</t>
         </is>
       </c>
       <c r="C577" t="inlineStr">
@@ -34951,24 +34988,24 @@
       </c>
       <c r="J577" t="inlineStr">
         <is>
-          <t>325</t>
+          <t>428</t>
         </is>
       </c>
     </row>
     <row r="578">
       <c r="A578" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>500 mb de R$ 109,90 por R$ 79,90 nos 2 primeiros meses.</t>
         </is>
       </c>
       <c r="B578" t="inlineStr">
         <is>
-          <t>1470</t>
+          <t>973</t>
         </is>
       </c>
       <c r="C578" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 0.00</t>
         </is>
       </c>
       <c r="D578" t="inlineStr">
@@ -35003,129 +35040,129 @@
       </c>
       <c r="J578" t="inlineStr">
         <is>
-          <t>846</t>
+          <t>325</t>
         </is>
       </c>
     </row>
     <row r="579">
       <c r="A579" t="inlineStr">
         <is>
+          <t>10% OFF</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>1470</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F579" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G579" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H579" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J579" t="inlineStr">
+        <is>
+          <t>846</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
           <t>Passagem + hospedagem + serviços terrestres***= 30% de desconto na compra do seguro.
 ***transfer, locação de carros e ingressos.</t>
         </is>
       </c>
-      <c r="B579" t="inlineStr">
+      <c r="B580" t="inlineStr">
         <is>
           <t>989</t>
         </is>
       </c>
-      <c r="C579" t="inlineStr">
+      <c r="C580" t="inlineStr">
         <is>
           <t>30.00%</t>
         </is>
       </c>
-      <c r="D579" t="inlineStr">
+      <c r="D580" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
-      <c r="E579" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F579" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G579" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H579" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I579" t="inlineStr">
+      <c r="E580" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F580" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G580" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H580" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I580" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J579" t="inlineStr">
+      <c r="J580" t="inlineStr">
         <is>
           <t>335</t>
-        </is>
-      </c>
-    </row>
-    <row r="580">
-      <c r="A580" t="inlineStr">
-        <is>
-          <t>100US$ DE DESCONTO</t>
-        </is>
-      </c>
-      <c r="B580" t="inlineStr">
-        <is>
-          <t>1425</t>
-        </is>
-      </c>
-      <c r="C580" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D580" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E580" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F580" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G580" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H580" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I580" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J580" t="inlineStr">
-        <is>
-          <t>797</t>
         </is>
       </c>
     </row>
     <row r="581">
       <c r="A581" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>100US$ DE DESCONTO</t>
         </is>
       </c>
       <c r="B581" t="inlineStr">
         <is>
-          <t>1532</t>
+          <t>1425</t>
         </is>
       </c>
       <c r="C581" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D581" t="inlineStr">
@@ -35160,19 +35197,19 @@
       </c>
       <c r="J581" t="inlineStr">
         <is>
-          <t>897</t>
+          <t>797</t>
         </is>
       </c>
     </row>
     <row r="582">
       <c r="A582" t="inlineStr">
         <is>
-          <t>Com este voucher você garante 10% de desconto em todos os serviços</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B582" t="inlineStr">
         <is>
-          <t>1168</t>
+          <t>1532</t>
         </is>
       </c>
       <c r="C582" t="inlineStr">
@@ -35212,24 +35249,24 @@
       </c>
       <c r="J582" t="inlineStr">
         <is>
-          <t>514</t>
+          <t>897</t>
         </is>
       </c>
     </row>
     <row r="583">
       <c r="A583" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 20% de desconto nas compras a partir de R$300,00.</t>
+          <t>Com este voucher você garante 10% de desconto em todos os serviços</t>
         </is>
       </c>
       <c r="B583" t="inlineStr">
         <is>
-          <t>1159</t>
+          <t>1168</t>
         </is>
       </c>
       <c r="C583" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D583" t="inlineStr">
@@ -35244,7 +35281,7 @@
       </c>
       <c r="F583" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G583" t="inlineStr">
@@ -35264,24 +35301,24 @@
       </c>
       <c r="J583" t="inlineStr">
         <is>
-          <t>553</t>
+          <t>514</t>
         </is>
       </c>
     </row>
     <row r="584">
       <c r="A584" t="inlineStr">
         <is>
-          <t>20% Off</t>
+          <t>Com este cupom você tem direito a 20% de desconto nas compras a partir de R$300,00.</t>
         </is>
       </c>
       <c r="B584" t="inlineStr">
         <is>
-          <t>1448</t>
+          <t>1159</t>
         </is>
       </c>
       <c r="C584" t="inlineStr">
         <is>
-          <t>12.00%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D584" t="inlineStr">
@@ -35296,7 +35333,7 @@
       </c>
       <c r="F584" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G584" t="inlineStr">
@@ -35316,24 +35353,24 @@
       </c>
       <c r="J584" t="inlineStr">
         <is>
-          <t>819</t>
+          <t>553</t>
         </is>
       </c>
     </row>
     <row r="585">
       <c r="A585" t="inlineStr">
         <is>
-          <t>Com este voucher você garante desconto de 15% nos óculos esportivos e casuais disponíveis na Brëll Óculos.</t>
+          <t>20% Off</t>
         </is>
       </c>
       <c r="B585" t="inlineStr">
         <is>
-          <t>1176</t>
+          <t>1448</t>
         </is>
       </c>
       <c r="C585" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>12.00%</t>
         </is>
       </c>
       <c r="D585" t="inlineStr">
@@ -35348,7 +35385,7 @@
       </c>
       <c r="F585" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G585" t="inlineStr">
@@ -35368,24 +35405,24 @@
       </c>
       <c r="J585" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>819</t>
         </is>
       </c>
     </row>
     <row r="586">
       <c r="A586" t="inlineStr">
         <is>
-          <t>Com este voucher você garante 10% de desconto em todos os planos não promocionais. Condição para pagamento PIX.</t>
+          <t>Com este voucher você garante desconto de 15% nos óculos esportivos e casuais disponíveis na Brëll Óculos.</t>
         </is>
       </c>
       <c r="B586" t="inlineStr">
         <is>
-          <t>1186</t>
+          <t>1176</t>
         </is>
       </c>
       <c r="C586" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D586" t="inlineStr">
@@ -35420,19 +35457,19 @@
       </c>
       <c r="J586" t="inlineStr">
         <is>
-          <t>531</t>
+          <t>520</t>
         </is>
       </c>
     </row>
     <row r="587">
       <c r="A587" t="inlineStr">
         <is>
-          <t>Garanta agora 10% de desconto utilizando o cupom exclusivo para Alunos Green.</t>
+          <t>Com este voucher você garante 10% de desconto em todos os planos não promocionais. Condição para pagamento PIX.</t>
         </is>
       </c>
       <c r="B587" t="inlineStr">
         <is>
-          <t>1116</t>
+          <t>1186</t>
         </is>
       </c>
       <c r="C587" t="inlineStr">
@@ -35452,7 +35489,7 @@
       </c>
       <c r="F587" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G587" t="inlineStr">
@@ -35472,24 +35509,24 @@
       </c>
       <c r="J587" t="inlineStr">
         <is>
-          <t>462</t>
+          <t>531</t>
         </is>
       </c>
     </row>
     <row r="588">
       <c r="A588" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 15% de desconto em todas as peças.</t>
+          <t>Garanta agora 10% de desconto utilizando o cupom exclusivo para Alunos Green.</t>
         </is>
       </c>
       <c r="B588" t="inlineStr">
         <is>
-          <t>1290</t>
+          <t>1116</t>
         </is>
       </c>
       <c r="C588" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D588" t="inlineStr">
@@ -35504,7 +35541,7 @@
       </c>
       <c r="F588" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G588" t="inlineStr">
@@ -35524,19 +35561,19 @@
       </c>
       <c r="J588" t="inlineStr">
         <is>
-          <t>634</t>
+          <t>462</t>
         </is>
       </c>
     </row>
     <row r="589">
       <c r="A589" t="inlineStr">
         <is>
-          <t>15% de desconto</t>
+          <t>Com este cupom você tem direito a 15% de desconto em todas as peças.</t>
         </is>
       </c>
       <c r="B589" t="inlineStr">
         <is>
-          <t>1089</t>
+          <t>1290</t>
         </is>
       </c>
       <c r="C589" t="inlineStr">
@@ -35556,7 +35593,7 @@
       </c>
       <c r="F589" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G589" t="inlineStr">
@@ -35576,24 +35613,24 @@
       </c>
       <c r="J589" t="inlineStr">
         <is>
-          <t>444</t>
+          <t>634</t>
         </is>
       </c>
     </row>
     <row r="590">
       <c r="A590" t="inlineStr">
         <is>
-          <t>20% nos aluguéis de vestidos de noivas , damas, pagens debutantes e nos acessórios fomos véus e grinaldas</t>
+          <t>15% de desconto</t>
         </is>
       </c>
       <c r="B590" t="inlineStr">
         <is>
-          <t>1070</t>
+          <t>1089</t>
         </is>
       </c>
       <c r="C590" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D590" t="inlineStr">
@@ -35608,7 +35645,7 @@
       </c>
       <c r="F590" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G590" t="inlineStr">
@@ -35628,12 +35665,64 @@
       </c>
       <c r="J590" t="inlineStr">
         <is>
-          <t>432</t>
+          <t>444</t>
         </is>
       </c>
     </row>
     <row r="591">
       <c r="A591" t="inlineStr">
+        <is>
+          <t>20% nos aluguéis de vestidos de noivas , damas, pagens debutantes e nos acessórios fomos véus e grinaldas</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>1070</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>20.00%</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F591" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G591" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H591" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I591" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J591" t="inlineStr">
+        <is>
+          <t>432</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
         <is>
           <t>Com este cupom na compra de um Iphone você ganha:
  - Fonte Turbo 20w 
@@ -35641,118 +35730,66 @@
  - Entrega Grátis</t>
         </is>
       </c>
-      <c r="B591" t="inlineStr">
+      <c r="B592" t="inlineStr">
         <is>
           <t>1147</t>
         </is>
       </c>
-      <c r="C591" t="inlineStr">
+      <c r="C592" t="inlineStr">
         <is>
           <t>R$ 0.00</t>
         </is>
       </c>
-      <c r="D591" t="inlineStr">
+      <c r="D592" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
-      <c r="E591" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F591" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G591" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H591" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I591" t="inlineStr">
+      <c r="E592" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F592" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G592" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H592" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I592" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J591" t="inlineStr">
+      <c r="J592" t="inlineStr">
         <is>
           <t>498</t>
-        </is>
-      </c>
-    </row>
-    <row r="592">
-      <c r="A592" t="inlineStr">
-        <is>
-          <t>Desconto de 20% em Psicoterapia individual.</t>
-        </is>
-      </c>
-      <c r="B592" t="inlineStr">
-        <is>
-          <t>1001</t>
-        </is>
-      </c>
-      <c r="C592" t="inlineStr">
-        <is>
-          <t>20.00%</t>
-        </is>
-      </c>
-      <c r="D592" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E592" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F592" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G592" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H592" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I592" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J592" t="inlineStr">
-        <is>
-          <t>343</t>
         </is>
       </c>
     </row>
     <row r="593">
       <c r="A593" t="inlineStr">
         <is>
-          <t>20% OFF</t>
+          <t>Desconto de 20% em Psicoterapia individual.</t>
         </is>
       </c>
       <c r="B593" t="inlineStr">
         <is>
-          <t>1609</t>
+          <t>1001</t>
         </is>
       </c>
       <c r="C593" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D593" t="inlineStr">
@@ -35762,7 +35799,7 @@
       </c>
       <c r="E593" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F593" t="inlineStr">
@@ -35782,29 +35819,29 @@
       </c>
       <c r="I593" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>Sem expiracao</t>
         </is>
       </c>
       <c r="J593" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>343</t>
         </is>
       </c>
     </row>
     <row r="594">
       <c r="A594" t="inlineStr">
         <is>
-          <t>15% de desconto nos serviços de cílios</t>
+          <t>20% OFF</t>
         </is>
       </c>
       <c r="B594" t="inlineStr">
         <is>
-          <t>997</t>
+          <t>1609</t>
         </is>
       </c>
       <c r="C594" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D594" t="inlineStr">
@@ -35814,7 +35851,7 @@
       </c>
       <c r="E594" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="F594" t="inlineStr">
@@ -35834,29 +35871,29 @@
       </c>
       <c r="I594" t="inlineStr">
         <is>
-          <t>Sem expiracao</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="J594" t="inlineStr">
         <is>
-          <t>341</t>
+          <t>961</t>
         </is>
       </c>
     </row>
     <row r="595">
       <c r="A595" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto em SIPAT para Empresas.</t>
+          <t>15% de desconto nos serviços de cílios</t>
         </is>
       </c>
       <c r="B595" t="inlineStr">
         <is>
-          <t>1280</t>
+          <t>997</t>
         </is>
       </c>
       <c r="C595" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D595" t="inlineStr">
@@ -35871,7 +35908,7 @@
       </c>
       <c r="F595" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G595" t="inlineStr">
@@ -35891,129 +35928,129 @@
       </c>
       <c r="J595" t="inlineStr">
         <is>
-          <t>608</t>
+          <t>341</t>
         </is>
       </c>
     </row>
     <row r="596">
       <c r="A596" t="inlineStr">
         <is>
+          <t>Com este cupom você tem direito a 10% de desconto em SIPAT para Empresas.</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>1280</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F596" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G596" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H596" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J596" t="inlineStr">
+        <is>
+          <t>608</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
           <t>10% em qualquer serviço 
 *Atendemos em domicilio!*</t>
         </is>
       </c>
-      <c r="B596" t="inlineStr">
+      <c r="B597" t="inlineStr">
         <is>
           <t>1029</t>
         </is>
       </c>
-      <c r="C596" t="inlineStr">
+      <c r="C597" t="inlineStr">
         <is>
           <t>10.00%</t>
         </is>
       </c>
-      <c r="D596" t="inlineStr">
+      <c r="D597" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
-      <c r="E596" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F596" t="inlineStr">
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F597" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G596" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H596" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I596" t="inlineStr">
+      <c r="G597" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H597" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I597" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J596" t="inlineStr">
+      <c r="J597" t="inlineStr">
         <is>
           <t>364</t>
-        </is>
-      </c>
-    </row>
-    <row r="597">
-      <c r="A597" t="inlineStr">
-        <is>
-          <t>Mais de R$ 350 reais em beneficios exclusivos</t>
-        </is>
-      </c>
-      <c r="B597" t="inlineStr">
-        <is>
-          <t>1605</t>
-        </is>
-      </c>
-      <c r="C597" t="inlineStr">
-        <is>
-          <t>R$ 350.00</t>
-        </is>
-      </c>
-      <c r="D597" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E597" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F597" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G597" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H597" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I597" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J597" t="inlineStr">
-        <is>
-          <t>957</t>
         </is>
       </c>
     </row>
     <row r="598">
       <c r="A598" t="inlineStr">
         <is>
-          <t>10% de desconto</t>
+          <t>Mais de R$ 350 reais em beneficios exclusivos</t>
         </is>
       </c>
       <c r="B598" t="inlineStr">
         <is>
-          <t>1068</t>
+          <t>1605</t>
         </is>
       </c>
       <c r="C598" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 350.00</t>
         </is>
       </c>
       <c r="D598" t="inlineStr">
@@ -36028,7 +36065,7 @@
       </c>
       <c r="F598" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G598" t="inlineStr">
@@ -36048,24 +36085,24 @@
       </c>
       <c r="J598" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>957</t>
         </is>
       </c>
     </row>
     <row r="599">
       <c r="A599" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 12% de desconto em cirurgias</t>
+          <t>10% de desconto</t>
         </is>
       </c>
       <c r="B599" t="inlineStr">
         <is>
-          <t>1256</t>
+          <t>1068</t>
         </is>
       </c>
       <c r="C599" t="inlineStr">
         <is>
-          <t>12.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D599" t="inlineStr">
@@ -36080,7 +36117,7 @@
       </c>
       <c r="F599" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G599" t="inlineStr">
@@ -36100,24 +36137,24 @@
       </c>
       <c r="J599" t="inlineStr">
         <is>
-          <t>590</t>
+          <t>430</t>
         </is>
       </c>
     </row>
     <row r="600">
       <c r="A600" t="inlineStr">
         <is>
-          <t>Com este voucher você garante 10% de desconto em todos os produtos da loja.</t>
+          <t>Com este cupom você tem direito a 12% de desconto em cirurgias</t>
         </is>
       </c>
       <c r="B600" t="inlineStr">
         <is>
-          <t>1164</t>
+          <t>1256</t>
         </is>
       </c>
       <c r="C600" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>12.00%</t>
         </is>
       </c>
       <c r="D600" t="inlineStr">
@@ -36152,24 +36189,24 @@
       </c>
       <c r="J600" t="inlineStr">
         <is>
-          <t>510</t>
+          <t>590</t>
         </is>
       </c>
     </row>
     <row r="601">
       <c r="A601" t="inlineStr">
         <is>
-          <t>Desconto de 20% em todos os tratamentos corporais e faciais não invasivos! Desconto não é válido para pacotes promocionais.</t>
+          <t>Com este voucher você garante 10% de desconto em todos os produtos da loja.</t>
         </is>
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>1298</t>
+          <t>1164</t>
         </is>
       </c>
       <c r="C601" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D601" t="inlineStr">
@@ -36204,24 +36241,24 @@
       </c>
       <c r="J601" t="inlineStr">
         <is>
-          <t>640</t>
+          <t>510</t>
         </is>
       </c>
     </row>
     <row r="602">
       <c r="A602" t="inlineStr">
         <is>
-          <t>5 marmitas + 5 sopas por apenas R$ 125,00</t>
+          <t>Desconto de 20% em todos os tratamentos corporais e faciais não invasivos! Desconto não é válido para pacotes promocionais.</t>
         </is>
       </c>
       <c r="B602" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1298</t>
         </is>
       </c>
       <c r="C602" t="inlineStr">
         <is>
-          <t>R$ 0.00</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D602" t="inlineStr">
@@ -36256,24 +36293,24 @@
       </c>
       <c r="J602" t="inlineStr">
         <is>
-          <t>342</t>
+          <t>640</t>
         </is>
       </c>
     </row>
     <row r="603">
       <c r="A603" t="inlineStr">
         <is>
-          <t>15% de descnto em produtos da loja.</t>
+          <t>5 marmitas + 5 sopas por apenas R$ 125,00</t>
         </is>
       </c>
       <c r="B603" t="inlineStr">
         <is>
-          <t>1335</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="C603" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>R$ 0.00</t>
         </is>
       </c>
       <c r="D603" t="inlineStr">
@@ -36288,7 +36325,7 @@
       </c>
       <c r="F603" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G603" t="inlineStr">
@@ -36308,24 +36345,24 @@
       </c>
       <c r="J603" t="inlineStr">
         <is>
-          <t>701</t>
+          <t>342</t>
         </is>
       </c>
     </row>
     <row r="604">
       <c r="A604" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 20% de desconto nos serviços de barba e cabelo.</t>
+          <t>15% de descnto em produtos da loja.</t>
         </is>
       </c>
       <c r="B604" t="inlineStr">
         <is>
-          <t>1245</t>
+          <t>1335</t>
         </is>
       </c>
       <c r="C604" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D604" t="inlineStr">
@@ -36360,24 +36397,24 @@
       </c>
       <c r="J604" t="inlineStr">
         <is>
-          <t>581</t>
+          <t>701</t>
         </is>
       </c>
     </row>
     <row r="605">
       <c r="A605" t="inlineStr">
         <is>
-          <t>10%OFF</t>
+          <t>Com este cupom você tem direito a 20% de desconto nos serviços de barba e cabelo.</t>
         </is>
       </c>
       <c r="B605" t="inlineStr">
         <is>
-          <t>1443</t>
+          <t>1245</t>
         </is>
       </c>
       <c r="C605" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D605" t="inlineStr">
@@ -36392,7 +36429,7 @@
       </c>
       <c r="F605" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G605" t="inlineStr">
@@ -36412,19 +36449,19 @@
       </c>
       <c r="J605" t="inlineStr">
         <is>
-          <t>815</t>
+          <t>581</t>
         </is>
       </c>
     </row>
     <row r="606">
       <c r="A606" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto para compras feitas através do nosso site.</t>
+          <t>10%OFF</t>
         </is>
       </c>
       <c r="B606" t="inlineStr">
         <is>
-          <t>1211</t>
+          <t>1443</t>
         </is>
       </c>
       <c r="C606" t="inlineStr">
@@ -36464,24 +36501,24 @@
       </c>
       <c r="J606" t="inlineStr">
         <is>
-          <t>556</t>
+          <t>815</t>
         </is>
       </c>
     </row>
     <row r="607">
       <c r="A607" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 20% de desconto para Kit Capa e película.</t>
+          <t>Com este cupom você tem direito a 10% de desconto para compras feitas através do nosso site.</t>
         </is>
       </c>
       <c r="B607" t="inlineStr">
         <is>
-          <t>1305</t>
+          <t>1211</t>
         </is>
       </c>
       <c r="C607" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D607" t="inlineStr">
@@ -36516,24 +36553,24 @@
       </c>
       <c r="J607" t="inlineStr">
         <is>
-          <t>648</t>
+          <t>556</t>
         </is>
       </c>
     </row>
     <row r="608">
       <c r="A608" t="inlineStr">
         <is>
-          <t>10% de desconto</t>
+          <t>Com este cupom você tem direito a 20% de desconto para Kit Capa e película.</t>
         </is>
       </c>
       <c r="B608" t="inlineStr">
         <is>
-          <t>1344</t>
+          <t>1305</t>
         </is>
       </c>
       <c r="C608" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D608" t="inlineStr">
@@ -36543,7 +36580,7 @@
       </c>
       <c r="E608" t="inlineStr">
         <is>
-          <t>-100</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F608" t="inlineStr">
@@ -36568,24 +36605,24 @@
       </c>
       <c r="J608" t="inlineStr">
         <is>
-          <t>716</t>
+          <t>648</t>
         </is>
       </c>
     </row>
     <row r="609">
       <c r="A609" t="inlineStr">
         <is>
-          <t>15% OFF CARMEL CUMBUCO</t>
+          <t>10% de desconto</t>
         </is>
       </c>
       <c r="B609" t="inlineStr">
         <is>
-          <t>1393</t>
+          <t>1344</t>
         </is>
       </c>
       <c r="C609" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D609" t="inlineStr">
@@ -36595,12 +36632,12 @@
       </c>
       <c r="E609" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>-100</t>
         </is>
       </c>
       <c r="F609" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G609" t="inlineStr">
@@ -36620,24 +36657,24 @@
       </c>
       <c r="J609" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>716</t>
         </is>
       </c>
     </row>
     <row r="610">
       <c r="A610" t="inlineStr">
         <is>
-          <t>10% Off no site</t>
+          <t>15% OFF CARMEL CUMBUCO</t>
         </is>
       </c>
       <c r="B610" t="inlineStr">
         <is>
-          <t>1568</t>
+          <t>1393</t>
         </is>
       </c>
       <c r="C610" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D610" t="inlineStr">
@@ -36652,7 +36689,7 @@
       </c>
       <c r="F610" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>21</t>
         </is>
       </c>
       <c r="G610" t="inlineStr">
@@ -36672,24 +36709,24 @@
       </c>
       <c r="J610" t="inlineStr">
         <is>
-          <t>927</t>
+          <t>110</t>
         </is>
       </c>
     </row>
     <row r="611">
       <c r="A611" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 50% de desconto em nossa consultoria de imagem</t>
+          <t>10% Off no site</t>
         </is>
       </c>
       <c r="B611" t="inlineStr">
         <is>
-          <t>1230</t>
+          <t>1568</t>
         </is>
       </c>
       <c r="C611" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D611" t="inlineStr">
@@ -36704,7 +36741,7 @@
       </c>
       <c r="F611" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G611" t="inlineStr">
@@ -36724,24 +36761,24 @@
       </c>
       <c r="J611" t="inlineStr">
         <is>
-          <t>574</t>
+          <t>927</t>
         </is>
       </c>
     </row>
     <row r="612">
       <c r="A612" t="inlineStr">
         <is>
-          <t>30%OFF</t>
+          <t>Com este cupom você tem direito a 50% de desconto em nossa consultoria de imagem</t>
         </is>
       </c>
       <c r="B612" t="inlineStr">
         <is>
-          <t>1446</t>
+          <t>1230</t>
         </is>
       </c>
       <c r="C612" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>50.00%</t>
         </is>
       </c>
       <c r="D612" t="inlineStr">
@@ -36756,7 +36793,7 @@
       </c>
       <c r="F612" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G612" t="inlineStr">
@@ -36776,24 +36813,24 @@
       </c>
       <c r="J612" t="inlineStr">
         <is>
-          <t>817</t>
+          <t>574</t>
         </is>
       </c>
     </row>
     <row r="613">
       <c r="A613" t="inlineStr">
         <is>
-          <t>15%OFF</t>
+          <t>30%OFF</t>
         </is>
       </c>
       <c r="B613" t="inlineStr">
         <is>
-          <t>1423</t>
+          <t>1446</t>
         </is>
       </c>
       <c r="C613" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D613" t="inlineStr">
@@ -36808,12 +36845,12 @@
       </c>
       <c r="F613" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G613" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H613" t="inlineStr">
@@ -36828,24 +36865,24 @@
       </c>
       <c r="J613" t="inlineStr">
         <is>
-          <t>796</t>
+          <t>817</t>
         </is>
       </c>
     </row>
     <row r="614">
       <c r="A614" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 20% de desconto no seu Óculos Sport.</t>
+          <t>15%OFF</t>
         </is>
       </c>
       <c r="B614" t="inlineStr">
         <is>
-          <t>1294</t>
+          <t>1423</t>
         </is>
       </c>
       <c r="C614" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D614" t="inlineStr">
@@ -36860,12 +36897,12 @@
       </c>
       <c r="F614" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>71</t>
         </is>
       </c>
       <c r="G614" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H614" t="inlineStr">
@@ -36880,24 +36917,24 @@
       </c>
       <c r="J614" t="inlineStr">
         <is>
-          <t>637</t>
+          <t>796</t>
         </is>
       </c>
     </row>
     <row r="615">
       <c r="A615" t="inlineStr">
         <is>
-          <t>15% OFF</t>
+          <t>Com este cupom você tem direito a 20% de desconto no seu Óculos Sport.</t>
         </is>
       </c>
       <c r="B615" t="inlineStr">
         <is>
-          <t>1375</t>
+          <t>1294</t>
         </is>
       </c>
       <c r="C615" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D615" t="inlineStr">
@@ -36912,7 +36949,7 @@
       </c>
       <c r="F615" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G615" t="inlineStr">
@@ -36932,24 +36969,24 @@
       </c>
       <c r="J615" t="inlineStr">
         <is>
-          <t>750</t>
+          <t>637</t>
         </is>
       </c>
     </row>
     <row r="616">
       <c r="A616" t="inlineStr">
         <is>
-          <t>Garanta agora 10% de desconto utilizando o cupom exclusivo para Alunos Green.</t>
+          <t>15% OFF</t>
         </is>
       </c>
       <c r="B616" t="inlineStr">
         <is>
-          <t>1114</t>
+          <t>1375</t>
         </is>
       </c>
       <c r="C616" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D616" t="inlineStr">
@@ -36964,7 +37001,7 @@
       </c>
       <c r="F616" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G616" t="inlineStr">
@@ -36984,129 +37021,129 @@
       </c>
       <c r="J616" t="inlineStr">
         <is>
-          <t>460</t>
+          <t>750</t>
         </is>
       </c>
     </row>
     <row r="617">
       <c r="A617" t="inlineStr">
         <is>
+          <t>Garanta agora 10% de desconto utilizando o cupom exclusivo para Alunos Green.</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>1114</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="G617" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H617" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I617" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J617" t="inlineStr">
+        <is>
+          <t>460</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
           <t>Com este cupom você tem direito a 10% de desconto em manutenção e reparos (trocar de telas,baterias,etc)
 Obs: Preços diferenciados para aquisição de aparelhos,air tags,alexa,etc..</t>
         </is>
       </c>
-      <c r="B617" t="inlineStr">
+      <c r="B618" t="inlineStr">
         <is>
           <t>1297</t>
         </is>
       </c>
-      <c r="C617" t="inlineStr">
+      <c r="C618" t="inlineStr">
         <is>
           <t>10.00%</t>
         </is>
       </c>
-      <c r="D617" t="inlineStr">
+      <c r="D618" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
-      <c r="E617" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F617" t="inlineStr">
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G617" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H617" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I617" t="inlineStr">
+      <c r="G618" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H618" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I618" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J617" t="inlineStr">
+      <c r="J618" t="inlineStr">
         <is>
           <t>639</t>
-        </is>
-      </c>
-    </row>
-    <row r="618">
-      <c r="A618" t="inlineStr">
-        <is>
-          <t>Com este cupom você tem direito a 10% de desconto no seu primeiro pedido.</t>
-        </is>
-      </c>
-      <c r="B618" t="inlineStr">
-        <is>
-          <t>1304</t>
-        </is>
-      </c>
-      <c r="C618" t="inlineStr">
-        <is>
-          <t>10.00%</t>
-        </is>
-      </c>
-      <c r="D618" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E618" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F618" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="G618" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H618" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I618" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J618" t="inlineStr">
-        <is>
-          <t>646</t>
         </is>
       </c>
     </row>
     <row r="619">
       <c r="A619" t="inlineStr">
         <is>
-          <t>4 sessões</t>
+          <t>Com este cupom você tem direito a 10% de desconto no seu primeiro pedido.</t>
         </is>
       </c>
       <c r="B619" t="inlineStr">
         <is>
-          <t>1590</t>
+          <t>1304</t>
         </is>
       </c>
       <c r="C619" t="inlineStr">
         <is>
-          <t>R$ 500.00</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D619" t="inlineStr">
@@ -37121,7 +37158,7 @@
       </c>
       <c r="F619" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G619" t="inlineStr">
@@ -37141,24 +37178,24 @@
       </c>
       <c r="J619" t="inlineStr">
         <is>
-          <t>943</t>
+          <t>646</t>
         </is>
       </c>
     </row>
     <row r="620">
       <c r="A620" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto em todo o nosso cardápio.</t>
+          <t>4 sessões</t>
         </is>
       </c>
       <c r="B620" t="inlineStr">
         <is>
-          <t>1241</t>
+          <t>1590</t>
         </is>
       </c>
       <c r="C620" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 500.00</t>
         </is>
       </c>
       <c r="D620" t="inlineStr">
@@ -37173,7 +37210,7 @@
       </c>
       <c r="F620" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G620" t="inlineStr">
@@ -37193,19 +37230,19 @@
       </c>
       <c r="J620" t="inlineStr">
         <is>
-          <t>579</t>
+          <t>943</t>
         </is>
       </c>
     </row>
     <row r="621">
       <c r="A621" t="inlineStr">
         <is>
-          <t>Garanta agora 10% de desconto no nosso COMBO de 10 refeições!</t>
+          <t>Com este cupom você tem direito a 10% de desconto em todo o nosso cardápio.</t>
         </is>
       </c>
       <c r="B621" t="inlineStr">
         <is>
-          <t>1103</t>
+          <t>1241</t>
         </is>
       </c>
       <c r="C621" t="inlineStr">
@@ -37225,7 +37262,7 @@
       </c>
       <c r="F621" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G621" t="inlineStr">
@@ -37245,19 +37282,19 @@
       </c>
       <c r="J621" t="inlineStr">
         <is>
-          <t>453</t>
+          <t>579</t>
         </is>
       </c>
     </row>
     <row r="622">
       <c r="A622" t="inlineStr">
         <is>
-          <t>Garanta agora 10% de desconto em nossa loja.</t>
+          <t>Garanta agora 10% de desconto no nosso COMBO de 10 refeições!</t>
         </is>
       </c>
       <c r="B622" t="inlineStr">
         <is>
-          <t>1302</t>
+          <t>1103</t>
         </is>
       </c>
       <c r="C622" t="inlineStr">
@@ -37277,7 +37314,7 @@
       </c>
       <c r="F622" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G622" t="inlineStr">
@@ -37297,287 +37334,287 @@
       </c>
       <c r="J622" t="inlineStr">
         <is>
-          <t>644</t>
+          <t>453</t>
         </is>
       </c>
     </row>
     <row r="623">
       <c r="A623" t="inlineStr">
         <is>
+          <t>Garanta agora 10% de desconto em nossa loja.</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>1302</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="G623" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H623" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J623" t="inlineStr">
+        <is>
+          <t>644</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
           <t>Com este cupom você tem direito a 10% de desconto no seu Óculo de Grau.
 Obs: Válido para primeira compra</t>
         </is>
       </c>
-      <c r="B623" t="inlineStr">
+      <c r="B624" t="inlineStr">
         <is>
           <t>1293</t>
         </is>
       </c>
-      <c r="C623" t="inlineStr">
+      <c r="C624" t="inlineStr">
         <is>
           <t>10.00%</t>
         </is>
       </c>
-      <c r="D623" t="inlineStr">
+      <c r="D624" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
-      <c r="E623" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F623" t="inlineStr">
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G623" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H623" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I623" t="inlineStr">
+      <c r="G624" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I624" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J623" t="inlineStr">
+      <c r="J624" t="inlineStr">
         <is>
           <t>637</t>
-        </is>
-      </c>
-    </row>
-    <row r="624">
-      <c r="A624" t="inlineStr">
-        <is>
-          <t>10% Off em serviços de cabelo</t>
-        </is>
-      </c>
-      <c r="B624" t="inlineStr">
-        <is>
-          <t>1577</t>
-        </is>
-      </c>
-      <c r="C624" t="inlineStr">
-        <is>
-          <t>10.00%</t>
-        </is>
-      </c>
-      <c r="D624" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E624" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F624" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G624" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H624" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I624" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J624" t="inlineStr">
-        <is>
-          <t>931</t>
         </is>
       </c>
     </row>
     <row r="625">
       <c r="A625" t="inlineStr">
         <is>
+          <t>10% Off em serviços de cabelo</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>1577</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F625" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G625" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H625" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J625" t="inlineStr">
+        <is>
+          <t>931</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
           <t>Você ganhou uma cortesia de 30 minutos de estúdio para gravar o seu contéudo.
 *Válido um por CPF</t>
         </is>
       </c>
-      <c r="B625" t="inlineStr">
+      <c r="B626" t="inlineStr">
         <is>
           <t>1244</t>
         </is>
       </c>
-      <c r="C625" t="inlineStr">
+      <c r="C626" t="inlineStr">
         <is>
           <t>R$ 0.00</t>
         </is>
       </c>
-      <c r="D625" t="inlineStr">
+      <c r="D626" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
-      <c r="E625" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F625" t="inlineStr">
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F626" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="G625" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H625" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I625" t="inlineStr">
+      <c r="G626" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H626" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I626" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J625" t="inlineStr">
+      <c r="J626" t="inlineStr">
         <is>
           <t>580</t>
         </is>
       </c>
     </row>
-    <row r="626">
-      <c r="A626" t="inlineStr">
+    <row r="627">
+      <c r="A627" t="inlineStr">
         <is>
           <t>Na primeira compra acima de R$50,00 ganhe 4 trufas língua de gato mil delícias
 *Exclusivo para loja do Shopping Iguatemi*</t>
         </is>
       </c>
-      <c r="B626" t="inlineStr">
+      <c r="B627" t="inlineStr">
         <is>
           <t>975</t>
         </is>
       </c>
-      <c r="C626" t="inlineStr">
+      <c r="C627" t="inlineStr">
         <is>
           <t>R$ 0.00</t>
         </is>
       </c>
-      <c r="D626" t="inlineStr">
+      <c r="D627" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
-      <c r="E626" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F626" t="inlineStr">
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F627" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="G626" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H626" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I626" t="inlineStr">
+      <c r="G627" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H627" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I627" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J626" t="inlineStr">
+      <c r="J627" t="inlineStr">
         <is>
           <t>326</t>
-        </is>
-      </c>
-    </row>
-    <row r="627">
-      <c r="A627" t="inlineStr">
-        <is>
-          <t>10% OFF</t>
-        </is>
-      </c>
-      <c r="B627" t="inlineStr">
-        <is>
-          <t>1512</t>
-        </is>
-      </c>
-      <c r="C627" t="inlineStr">
-        <is>
-          <t>10.00%</t>
-        </is>
-      </c>
-      <c r="D627" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E627" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F627" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="G627" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H627" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I627" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J627" t="inlineStr">
-        <is>
-          <t>878</t>
         </is>
       </c>
     </row>
     <row r="628">
       <c r="A628" t="inlineStr">
         <is>
-          <t>Clientes novos ganha 1 sessão de massagem relaxante e 3 sessões de depilação nas axilas</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B628" t="inlineStr">
         <is>
-          <t>1013</t>
+          <t>1512</t>
         </is>
       </c>
       <c r="C628" t="inlineStr">
         <is>
-          <t>R$ 0.00</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D628" t="inlineStr">
@@ -37592,7 +37629,7 @@
       </c>
       <c r="F628" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G628" t="inlineStr">
@@ -37612,24 +37649,24 @@
       </c>
       <c r="J628" t="inlineStr">
         <is>
-          <t>353</t>
+          <t>878</t>
         </is>
       </c>
     </row>
     <row r="629">
       <c r="A629" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto em nossos produtos.</t>
+          <t>Clientes novos ganha 1 sessão de massagem relaxante e 3 sessões de depilação nas axilas</t>
         </is>
       </c>
       <c r="B629" t="inlineStr">
         <is>
-          <t>1292</t>
+          <t>1013</t>
         </is>
       </c>
       <c r="C629" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 0.00</t>
         </is>
       </c>
       <c r="D629" t="inlineStr">
@@ -37644,7 +37681,7 @@
       </c>
       <c r="F629" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G629" t="inlineStr">
@@ -37664,124 +37701,124 @@
       </c>
       <c r="J629" t="inlineStr">
         <is>
-          <t>636</t>
+          <t>353</t>
         </is>
       </c>
     </row>
     <row r="630">
       <c r="A630" t="inlineStr">
         <is>
+          <t>Com este cupom você tem direito a 10% de desconto em nossos produtos.</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>1292</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F630" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G630" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H630" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J630" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
           <t>Desconto dentro do app da Schon com o nome “Schon Green”
 Baixe o APP SCHON e tenha acesso ao desconto do parceiro.</t>
         </is>
       </c>
-      <c r="B630" t="inlineStr">
+      <c r="B631" t="inlineStr">
         <is>
           <t>1288</t>
         </is>
       </c>
-      <c r="C630" t="inlineStr">
+      <c r="C631" t="inlineStr">
         <is>
           <t>R$ 0.00</t>
         </is>
       </c>
-      <c r="D630" t="inlineStr">
+      <c r="D631" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
-      <c r="E630" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F630" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G630" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H630" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I630" t="inlineStr">
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F631" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G631" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H631" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I631" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J630" t="inlineStr">
+      <c r="J631" t="inlineStr">
         <is>
           <t>619</t>
-        </is>
-      </c>
-    </row>
-    <row r="631">
-      <c r="A631" t="inlineStr">
-        <is>
-          <t>Com este cupom você tem direito a 10% de desconto em nosso cardápio.</t>
-        </is>
-      </c>
-      <c r="B631" t="inlineStr">
-        <is>
-          <t>1207</t>
-        </is>
-      </c>
-      <c r="C631" t="inlineStr">
-        <is>
-          <t>10.00%</t>
-        </is>
-      </c>
-      <c r="D631" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E631" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F631" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="G631" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H631" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I631" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J631" t="inlineStr">
-        <is>
-          <t>547</t>
         </is>
       </c>
     </row>
     <row r="632">
       <c r="A632" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>Com este cupom você tem direito a 10% de desconto em nosso cardápio.</t>
         </is>
       </c>
       <c r="B632" t="inlineStr">
         <is>
-          <t>1530</t>
+          <t>1207</t>
         </is>
       </c>
       <c r="C632" t="inlineStr">
@@ -37801,7 +37838,7 @@
       </c>
       <c r="F632" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G632" t="inlineStr">
@@ -37821,129 +37858,129 @@
       </c>
       <c r="J632" t="inlineStr">
         <is>
-          <t>896</t>
+          <t>547</t>
         </is>
       </c>
     </row>
     <row r="633">
       <c r="A633" t="inlineStr">
         <is>
+          <t>10% OFF</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>1530</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F633" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G633" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H633" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I633" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J633" t="inlineStr">
+        <is>
+          <t>896</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
           <t>Garanta 15% de desconto no valor do curso.
 *Não incluso a taxa de matrícula e o material.</t>
         </is>
       </c>
-      <c r="B633" t="inlineStr">
+      <c r="B634" t="inlineStr">
         <is>
           <t>1093</t>
         </is>
       </c>
-      <c r="C633" t="inlineStr">
+      <c r="C634" t="inlineStr">
         <is>
           <t>15.00%</t>
         </is>
       </c>
-      <c r="D633" t="inlineStr">
+      <c r="D634" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
-      <c r="E633" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F633" t="inlineStr">
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F634" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G633" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H633" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I633" t="inlineStr">
+      <c r="G634" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H634" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I634" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J633" t="inlineStr">
+      <c r="J634" t="inlineStr">
         <is>
           <t>447</t>
-        </is>
-      </c>
-    </row>
-    <row r="634">
-      <c r="A634" t="inlineStr">
-        <is>
-          <t>Com este cupom você tem direio a 20% de desconto nas compras acima de R$400,00</t>
-        </is>
-      </c>
-      <c r="B634" t="inlineStr">
-        <is>
-          <t>1076</t>
-        </is>
-      </c>
-      <c r="C634" t="inlineStr">
-        <is>
-          <t>20.00%</t>
-        </is>
-      </c>
-      <c r="D634" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E634" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F634" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="G634" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H634" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I634" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J634" t="inlineStr">
-        <is>
-          <t>625</t>
         </is>
       </c>
     </row>
     <row r="635">
       <c r="A635" t="inlineStr">
         <is>
-          <t>Sessão Integrativa</t>
+          <t>Com este cupom você tem direio a 20% de desconto nas compras acima de R$400,00</t>
         </is>
       </c>
       <c r="B635" t="inlineStr">
         <is>
-          <t>1588</t>
+          <t>1076</t>
         </is>
       </c>
       <c r="C635" t="inlineStr">
         <is>
-          <t>R$ 120.00</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D635" t="inlineStr">
@@ -37958,7 +37995,7 @@
       </c>
       <c r="F635" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G635" t="inlineStr">
@@ -37978,24 +38015,24 @@
       </c>
       <c r="J635" t="inlineStr">
         <is>
-          <t>943</t>
+          <t>625</t>
         </is>
       </c>
     </row>
     <row r="636">
       <c r="A636" t="inlineStr">
         <is>
-          <t>10% de desconto</t>
+          <t>Sessão Integrativa</t>
         </is>
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>979</t>
+          <t>1588</t>
         </is>
       </c>
       <c r="C636" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 120.00</t>
         </is>
       </c>
       <c r="D636" t="inlineStr">
@@ -38010,7 +38047,7 @@
       </c>
       <c r="F636" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G636" t="inlineStr">
@@ -38030,19 +38067,19 @@
       </c>
       <c r="J636" t="inlineStr">
         <is>
-          <t>329</t>
+          <t>943</t>
         </is>
       </c>
     </row>
     <row r="637">
       <c r="A637" t="inlineStr">
         <is>
-          <t>10% de desconto na consulta presencial com retorno. 10% de desconto na consulta on-line sem retorno.</t>
+          <t>10% de desconto</t>
         </is>
       </c>
       <c r="B637" t="inlineStr">
         <is>
-          <t>1180</t>
+          <t>979</t>
         </is>
       </c>
       <c r="C637" t="inlineStr">
@@ -38062,7 +38099,7 @@
       </c>
       <c r="F637" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G637" t="inlineStr">
@@ -38082,19 +38119,19 @@
       </c>
       <c r="J637" t="inlineStr">
         <is>
-          <t>524</t>
+          <t>329</t>
         </is>
       </c>
     </row>
     <row r="638">
       <c r="A638" t="inlineStr">
         <is>
-          <t>10%OFF</t>
+          <t>10% de desconto na consulta presencial com retorno. 10% de desconto na consulta on-line sem retorno.</t>
         </is>
       </c>
       <c r="B638" t="inlineStr">
         <is>
-          <t>1418</t>
+          <t>1180</t>
         </is>
       </c>
       <c r="C638" t="inlineStr">
@@ -38114,7 +38151,7 @@
       </c>
       <c r="F638" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G638" t="inlineStr">
@@ -38134,129 +38171,129 @@
       </c>
       <c r="J638" t="inlineStr">
         <is>
-          <t>791</t>
+          <t>524</t>
         </is>
       </c>
     </row>
     <row r="639">
       <c r="A639" t="inlineStr">
         <is>
+          <t>10%OFF</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>1418</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F639" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="G639" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H639" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I639" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J639" t="inlineStr">
+        <is>
+          <t>791</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
           <t>Assessorias de RH
 Garanta agora 10% de desconto em Presencial ou online</t>
         </is>
       </c>
-      <c r="B639" t="inlineStr">
+      <c r="B640" t="inlineStr">
         <is>
           <t>1318</t>
         </is>
       </c>
-      <c r="C639" t="inlineStr">
+      <c r="C640" t="inlineStr">
         <is>
           <t>10.00%</t>
         </is>
       </c>
-      <c r="D639" t="inlineStr">
+      <c r="D640" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
-      <c r="E639" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F639" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G639" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H639" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I639" t="inlineStr">
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F640" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G640" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H640" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I640" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J639" t="inlineStr">
+      <c r="J640" t="inlineStr">
         <is>
           <t>656</t>
-        </is>
-      </c>
-    </row>
-    <row r="640">
-      <c r="A640" t="inlineStr">
-        <is>
-          <t>30% de desconto em serviços , alinhamento e balanceamento</t>
-        </is>
-      </c>
-      <c r="B640" t="inlineStr">
-        <is>
-          <t>993</t>
-        </is>
-      </c>
-      <c r="C640" t="inlineStr">
-        <is>
-          <t>30.00%</t>
-        </is>
-      </c>
-      <c r="D640" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E640" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F640" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G640" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H640" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I640" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J640" t="inlineStr">
-        <is>
-          <t>338</t>
         </is>
       </c>
     </row>
     <row r="641">
       <c r="A641" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>30% de desconto em serviços , alinhamento e balanceamento</t>
         </is>
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>1410</t>
+          <t>993</t>
         </is>
       </c>
       <c r="C641" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>30.00%</t>
         </is>
       </c>
       <c r="D641" t="inlineStr">
@@ -38271,7 +38308,7 @@
       </c>
       <c r="F641" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G641" t="inlineStr">
@@ -38291,19 +38328,19 @@
       </c>
       <c r="J641" t="inlineStr">
         <is>
-          <t>781</t>
+          <t>338</t>
         </is>
       </c>
     </row>
     <row r="642">
       <c r="A642" t="inlineStr">
         <is>
-          <t>10%OFF</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>1442</t>
+          <t>1410</t>
         </is>
       </c>
       <c r="C642" t="inlineStr">
@@ -38323,7 +38360,7 @@
       </c>
       <c r="F642" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G642" t="inlineStr">
@@ -38343,24 +38380,24 @@
       </c>
       <c r="J642" t="inlineStr">
         <is>
-          <t>813</t>
+          <t>781</t>
         </is>
       </c>
     </row>
     <row r="643">
       <c r="A643" t="inlineStr">
         <is>
-          <t>15% OFF</t>
+          <t>10%OFF</t>
         </is>
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>1559</t>
+          <t>1442</t>
         </is>
       </c>
       <c r="C643" t="inlineStr">
         <is>
-          <t>14.98%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D643" t="inlineStr">
@@ -38375,12 +38412,12 @@
       </c>
       <c r="F643" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G643" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H643" t="inlineStr">
@@ -38395,24 +38432,24 @@
       </c>
       <c r="J643" t="inlineStr">
         <is>
-          <t>915</t>
+          <t>813</t>
         </is>
       </c>
     </row>
     <row r="644">
       <c r="A644" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto nos produtos da nossa loja online.</t>
+          <t>15% OFF</t>
         </is>
       </c>
       <c r="B644" t="inlineStr">
         <is>
-          <t>1139</t>
+          <t>1559</t>
         </is>
       </c>
       <c r="C644" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>14.98%</t>
         </is>
       </c>
       <c r="D644" t="inlineStr">
@@ -38427,12 +38464,12 @@
       </c>
       <c r="F644" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G644" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H644" t="inlineStr">
@@ -38447,24 +38484,24 @@
       </c>
       <c r="J644" t="inlineStr">
         <is>
-          <t>492</t>
+          <t>915</t>
         </is>
       </c>
     </row>
     <row r="645">
       <c r="A645" t="inlineStr">
         <is>
-          <t>17% de desconto em 2024</t>
+          <t>Com este cupom você tem direito a 10% de desconto nos produtos da nossa loja online.</t>
         </is>
       </c>
       <c r="B645" t="inlineStr">
         <is>
-          <t>1327</t>
+          <t>1139</t>
         </is>
       </c>
       <c r="C645" t="inlineStr">
         <is>
-          <t>17.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D645" t="inlineStr">
@@ -38479,7 +38516,7 @@
       </c>
       <c r="F645" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G645" t="inlineStr">
@@ -38499,182 +38536,182 @@
       </c>
       <c r="J645" t="inlineStr">
         <is>
-          <t>663</t>
+          <t>492</t>
         </is>
       </c>
     </row>
     <row r="646">
       <c r="A646" t="inlineStr">
         <is>
+          <t>17% de desconto em 2024</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>1327</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>17.00%</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G646" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H646" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I646" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J646" t="inlineStr">
+        <is>
+          <t>663</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
           <t>Com este cupom você tem direito a 20% de desconto em todos os serviços.
 Trabalhamos com contrato de manutenção e serviços avulsos.</t>
         </is>
       </c>
-      <c r="B646" t="inlineStr">
+      <c r="B647" t="inlineStr">
         <is>
           <t>1225</t>
         </is>
       </c>
-      <c r="C646" t="inlineStr">
+      <c r="C647" t="inlineStr">
         <is>
           <t>20.00%</t>
         </is>
       </c>
-      <c r="D646" t="inlineStr">
+      <c r="D647" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
-      <c r="E646" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F646" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G646" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H646" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I646" t="inlineStr">
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G647" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H647" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I647" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J646" t="inlineStr">
+      <c r="J647" t="inlineStr">
         <is>
           <t>566</t>
         </is>
       </c>
     </row>
-    <row r="647">
-      <c r="A647" t="inlineStr">
+    <row r="648">
+      <c r="A648" t="inlineStr">
         <is>
           <t>Com este cupom você tem direito a 6% de descontos em nossas peças!
 Obs: Válido para pagamento no crédito.</t>
         </is>
       </c>
-      <c r="B647" t="inlineStr">
+      <c r="B648" t="inlineStr">
         <is>
           <t>1223</t>
         </is>
       </c>
-      <c r="C647" t="inlineStr">
+      <c r="C648" t="inlineStr">
         <is>
           <t>6.00%</t>
         </is>
       </c>
-      <c r="D647" t="inlineStr">
+      <c r="D648" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
-      <c r="E647" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F647" t="inlineStr">
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G647" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H647" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I647" t="inlineStr">
+      <c r="G648" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H648" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I648" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J647" t="inlineStr">
+      <c r="J648" t="inlineStr">
         <is>
           <t>563</t>
-        </is>
-      </c>
-    </row>
-    <row r="648">
-      <c r="A648" t="inlineStr">
-        <is>
-          <t>15% de desconto</t>
-        </is>
-      </c>
-      <c r="B648" t="inlineStr">
-        <is>
-          <t>1072</t>
-        </is>
-      </c>
-      <c r="C648" t="inlineStr">
-        <is>
-          <t>15.00%</t>
-        </is>
-      </c>
-      <c r="D648" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E648" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F648" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G648" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H648" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I648" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J648" t="inlineStr">
-        <is>
-          <t>434</t>
         </is>
       </c>
     </row>
     <row r="649">
       <c r="A649" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>15% de desconto</t>
         </is>
       </c>
       <c r="B649" t="inlineStr">
         <is>
-          <t>1586</t>
+          <t>1072</t>
         </is>
       </c>
       <c r="C649" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D649" t="inlineStr">
@@ -38689,7 +38726,7 @@
       </c>
       <c r="F649" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G649" t="inlineStr">
@@ -38709,19 +38746,19 @@
       </c>
       <c r="J649" t="inlineStr">
         <is>
-          <t>941</t>
+          <t>434</t>
         </is>
       </c>
     </row>
     <row r="650">
       <c r="A650" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto nas suas tatoos.</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>1080</t>
+          <t>1586</t>
         </is>
       </c>
       <c r="C650" t="inlineStr">
@@ -38741,7 +38778,7 @@
       </c>
       <c r="F650" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G650" t="inlineStr">
@@ -38761,19 +38798,19 @@
       </c>
       <c r="J650" t="inlineStr">
         <is>
-          <t>630</t>
+          <t>941</t>
         </is>
       </c>
     </row>
     <row r="651">
       <c r="A651" t="inlineStr">
         <is>
-          <t>10% Off</t>
+          <t>Com este cupom você tem direito a 10% de desconto nas suas tatoos.</t>
         </is>
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>1342</t>
+          <t>1080</t>
         </is>
       </c>
       <c r="C651" t="inlineStr">
@@ -38793,7 +38830,7 @@
       </c>
       <c r="F651" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G651" t="inlineStr">
@@ -38813,24 +38850,24 @@
       </c>
       <c r="J651" t="inlineStr">
         <is>
-          <t>714</t>
+          <t>630</t>
         </is>
       </c>
     </row>
     <row r="652">
       <c r="A652" t="inlineStr">
         <is>
-          <t>20% off</t>
+          <t>10% Off</t>
         </is>
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>1607</t>
+          <t>1342</t>
         </is>
       </c>
       <c r="C652" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D652" t="inlineStr">
@@ -38845,7 +38882,7 @@
       </c>
       <c r="F652" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>67</t>
         </is>
       </c>
       <c r="G652" t="inlineStr">
@@ -38865,24 +38902,24 @@
       </c>
       <c r="J652" t="inlineStr">
         <is>
-          <t>959</t>
+          <t>714</t>
         </is>
       </c>
     </row>
     <row r="653">
       <c r="A653" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>20% off</t>
         </is>
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t>1498</t>
+          <t>1607</t>
         </is>
       </c>
       <c r="C653" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="D653" t="inlineStr">
@@ -38897,7 +38934,7 @@
       </c>
       <c r="F653" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G653" t="inlineStr">
@@ -38917,24 +38954,24 @@
       </c>
       <c r="J653" t="inlineStr">
         <is>
-          <t>871</t>
+          <t>959</t>
         </is>
       </c>
     </row>
     <row r="654">
       <c r="A654" t="inlineStr">
         <is>
-          <t>Frete grátis nas compras acima de 50 reais.</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B654" t="inlineStr">
         <is>
-          <t>1055</t>
+          <t>1498</t>
         </is>
       </c>
       <c r="C654" t="inlineStr">
         <is>
-          <t>R$ 0.00</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D654" t="inlineStr">
@@ -38949,7 +38986,7 @@
       </c>
       <c r="F654" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G654" t="inlineStr">
@@ -38969,24 +39006,24 @@
       </c>
       <c r="J654" t="inlineStr">
         <is>
-          <t>418</t>
+          <t>871</t>
         </is>
       </c>
     </row>
     <row r="655">
       <c r="A655" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>Frete grátis nas compras acima de 50 reais.</t>
         </is>
       </c>
       <c r="B655" t="inlineStr">
         <is>
-          <t>1539</t>
+          <t>1055</t>
         </is>
       </c>
       <c r="C655" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 0.00</t>
         </is>
       </c>
       <c r="D655" t="inlineStr">
@@ -39021,19 +39058,19 @@
       </c>
       <c r="J655" t="inlineStr">
         <is>
-          <t>906</t>
+          <t>418</t>
         </is>
       </c>
     </row>
     <row r="656">
       <c r="A656" t="inlineStr">
         <is>
-          <t>10% de desconto</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B656" t="inlineStr">
         <is>
-          <t>1355</t>
+          <t>1539</t>
         </is>
       </c>
       <c r="C656" t="inlineStr">
@@ -39053,7 +39090,7 @@
       </c>
       <c r="F656" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G656" t="inlineStr">
@@ -39073,24 +39110,24 @@
       </c>
       <c r="J656" t="inlineStr">
         <is>
-          <t>737</t>
+          <t>906</t>
         </is>
       </c>
     </row>
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>15% de desconto ( não válido às sextas e sábados)</t>
+          <t>10% de desconto</t>
         </is>
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>1026</t>
+          <t>1355</t>
         </is>
       </c>
       <c r="C657" t="inlineStr">
         <is>
-          <t>15.00%</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D657" t="inlineStr">
@@ -39105,7 +39142,7 @@
       </c>
       <c r="F657" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G657" t="inlineStr">
@@ -39125,19 +39162,19 @@
       </c>
       <c r="J657" t="inlineStr">
         <is>
-          <t>361</t>
+          <t>737</t>
         </is>
       </c>
     </row>
     <row r="658">
       <c r="A658" t="inlineStr">
         <is>
-          <t>15% de desconto nos serviços de cílios e design de sobrancelhas</t>
+          <t>15% de desconto ( não válido às sextas e sábados)</t>
         </is>
       </c>
       <c r="B658" t="inlineStr">
         <is>
-          <t>995</t>
+          <t>1026</t>
         </is>
       </c>
       <c r="C658" t="inlineStr">
@@ -39157,7 +39194,7 @@
       </c>
       <c r="F658" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G658" t="inlineStr">
@@ -39177,24 +39214,24 @@
       </c>
       <c r="J658" t="inlineStr">
         <is>
-          <t>340</t>
+          <t>361</t>
         </is>
       </c>
     </row>
     <row r="659">
       <c r="A659" t="inlineStr">
         <is>
-          <t>A cada 1 real gasto na loja é convertido em ponto e o aluno poderá acumular ou usar de imediato.</t>
+          <t>15% de desconto nos serviços de cílios e design de sobrancelhas</t>
         </is>
       </c>
       <c r="B659" t="inlineStr">
         <is>
-          <t>1188</t>
+          <t>995</t>
         </is>
       </c>
       <c r="C659" t="inlineStr">
         <is>
-          <t>R$ 0.00</t>
+          <t>15.00%</t>
         </is>
       </c>
       <c r="D659" t="inlineStr">
@@ -39229,24 +39266,24 @@
       </c>
       <c r="J659" t="inlineStr">
         <is>
-          <t>532</t>
+          <t>340</t>
         </is>
       </c>
     </row>
     <row r="660">
       <c r="A660" t="inlineStr">
         <is>
-          <t>10% OFF</t>
+          <t>A cada 1 real gasto na loja é convertido em ponto e o aluno poderá acumular ou usar de imediato.</t>
         </is>
       </c>
       <c r="B660" t="inlineStr">
         <is>
-          <t>1515</t>
+          <t>1188</t>
         </is>
       </c>
       <c r="C660" t="inlineStr">
         <is>
-          <t>10.00%</t>
+          <t>R$ 0.00</t>
         </is>
       </c>
       <c r="D660" t="inlineStr">
@@ -39281,24 +39318,24 @@
       </c>
       <c r="J660" t="inlineStr">
         <is>
-          <t>881</t>
+          <t>532</t>
         </is>
       </c>
     </row>
     <row r="661">
       <c r="A661" t="inlineStr">
         <is>
-          <t>Avaliação Facial Personalizada com IA</t>
+          <t>10% OFF</t>
         </is>
       </c>
       <c r="B661" t="inlineStr">
         <is>
-          <t>1500</t>
+          <t>1515</t>
         </is>
       </c>
       <c r="C661" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10.00%</t>
         </is>
       </c>
       <c r="D661" t="inlineStr">
@@ -39313,7 +39350,7 @@
       </c>
       <c r="F661" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G661" t="inlineStr">
@@ -39333,124 +39370,124 @@
       </c>
       <c r="J661" t="inlineStr">
         <is>
-          <t>873</t>
+          <t>881</t>
         </is>
       </c>
     </row>
     <row r="662">
       <c r="A662" t="inlineStr">
         <is>
+          <t>Avaliação Facial Personalizada com IA</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>1500</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F662" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G662" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H662" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J662" t="inlineStr">
+        <is>
+          <t>873</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
           <t>15% de desconto (não é válido para joias em promoção, alianças, relógios e best seller)
 Válido apenas na loja do Riomar Papicu.</t>
         </is>
       </c>
-      <c r="B662" t="inlineStr">
+      <c r="B663" t="inlineStr">
         <is>
           <t>1320</t>
         </is>
       </c>
-      <c r="C662" t="inlineStr">
+      <c r="C663" t="inlineStr">
         <is>
           <t>15.00%</t>
         </is>
       </c>
-      <c r="D662" t="inlineStr">
+      <c r="D663" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
-      <c r="E662" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F662" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G662" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H662" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I662" t="inlineStr">
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G663" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H663" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I663" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J662" t="inlineStr">
+      <c r="J663" t="inlineStr">
         <is>
           <t>657</t>
-        </is>
-      </c>
-    </row>
-    <row r="663">
-      <c r="A663" t="inlineStr">
-        <is>
-          <t>10% de desconto em todos os produtos da loja. Válido apenas para pagamentos por cartão de credito.</t>
-        </is>
-      </c>
-      <c r="B663" t="inlineStr">
-        <is>
-          <t>1191</t>
-        </is>
-      </c>
-      <c r="C663" t="inlineStr">
-        <is>
-          <t>10.00%</t>
-        </is>
-      </c>
-      <c r="D663" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-      <c r="E663" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F663" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G663" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H663" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I663" t="inlineStr">
-        <is>
-          <t>Sem expiracao</t>
-        </is>
-      </c>
-      <c r="J663" t="inlineStr">
-        <is>
-          <t>533</t>
         </is>
       </c>
     </row>
     <row r="664">
       <c r="A664" t="inlineStr">
         <is>
-          <t>10% de desconto em qualquer produto (lentes e armações)</t>
+          <t>10% de desconto em todos os produtos da loja. Válido apenas para pagamentos por cartão de credito.</t>
         </is>
       </c>
       <c r="B664" t="inlineStr">
         <is>
-          <t>1014</t>
+          <t>1191</t>
         </is>
       </c>
       <c r="C664" t="inlineStr">
@@ -39490,19 +39527,19 @@
       </c>
       <c r="J664" t="inlineStr">
         <is>
-          <t>354</t>
+          <t>533</t>
         </is>
       </c>
     </row>
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Com este cupom você tem direito a 10% de desconto nas suas compras.</t>
+          <t>10% de desconto em qualquer produto (lentes e armações)</t>
         </is>
       </c>
       <c r="B665" t="inlineStr">
         <is>
-          <t>1131</t>
+          <t>1014</t>
         </is>
       </c>
       <c r="C665" t="inlineStr">
@@ -39542,66 +39579,118 @@
       </c>
       <c r="J665" t="inlineStr">
         <is>
-          <t>484</t>
+          <t>354</t>
         </is>
       </c>
     </row>
     <row r="666">
       <c r="A666" t="inlineStr">
         <is>
+          <t>Com este cupom você tem direito a 10% de desconto nas suas compras.</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>1131</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G666" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H666" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I666" t="inlineStr">
+        <is>
+          <t>Sem expiracao</t>
+        </is>
+      </c>
+      <c r="J666" t="inlineStr">
+        <is>
+          <t>484</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
           <t>Com este cupom você tem direito a 20% de desconto nas compras em nossa loja.</t>
         </is>
       </c>
-      <c r="B666" t="inlineStr">
+      <c r="B667" t="inlineStr">
         <is>
           <t>1125</t>
         </is>
       </c>
-      <c r="C666" t="inlineStr">
+      <c r="C667" t="inlineStr">
         <is>
           <t>20.00%</t>
         </is>
       </c>
-      <c r="D666" t="inlineStr">
+      <c r="D667" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
-      <c r="E666" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F666" t="inlineStr">
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G666" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H666" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I666" t="inlineStr">
+      <c r="G667" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H667" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I667" t="inlineStr">
         <is>
           <t>Sem expiracao</t>
         </is>
       </c>
-      <c r="J666" t="inlineStr">
+      <c r="J667" t="inlineStr">
         <is>
           <t>478</t>
         </is>
       </c>
     </row>
-    <row r="668">
-      <c r="A668" t="inlineStr">
-        <is>
-          <t>Atualizado: 02/10/2026 13:02 | Ativas: 849 | Inativas: 0</t>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>Atualizado: 03/10/2026 11:29 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -39616,7 +39705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E714"/>
+  <dimension ref="A1:E715"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -58642,10 +58731,37 @@
         <v>18</v>
       </c>
     </row>
-    <row r="714">
-      <c r="A714" t="inlineStr">
-        <is>
-          <t>Atualizado: 02/10/2026 13:02 | Total: 711 | c/ usuario: 196 | s/ usuario: 515</t>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>975</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>Raízes Natuá</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>Heloá Jurgutis de Paula / raizesnatua@gmail.com</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>ALIMENTAÇÃO</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>Atualizado: 03/10/2026 11:29 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -58660,7 +58776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C747"/>
+  <dimension ref="A1:C748"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68351,16 +68467,29 @@
         </is>
       </c>
       <c r="B745" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C745" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="747">
-      <c r="A747" t="inlineStr">
-        <is>
-          <t>Atualizado: 02/10/2026 13:02 | Total dias: 744</t>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B746" t="n">
+        <v>1</v>
+      </c>
+      <c r="C746" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>Atualizado: 03/10/2026 11:29 | Total dias: 745</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-04 15:06 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G117"/>
+  <dimension ref="A1:G118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4775,6 +4775,43 @@
         </is>
       </c>
       <c r="G117" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>04/10/2026 12:03</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>6633</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>187</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -5569,7 +5606,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -6094,7 +6131,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -8075,7 +8112,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -24264,7 +24301,7 @@
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G372" t="inlineStr">
@@ -31001,7 +31038,7 @@
       </c>
       <c r="F501" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G501" t="inlineStr">
@@ -36897,7 +36934,7 @@
       </c>
       <c r="F614" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>72</t>
         </is>
       </c>
       <c r="G614" t="inlineStr">
@@ -39690,7 +39727,7 @@
     <row r="669">
       <c r="A669" t="inlineStr">
         <is>
-          <t>Atualizado: 03/10/2026 11:29 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 04/10/2026 12:03 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -58761,7 +58798,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 03/10/2026 11:29 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 04/10/2026 12:03 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -68480,7 +68517,7 @@
         </is>
       </c>
       <c r="B746" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C746" t="n">
         <v>0</v>
@@ -68489,7 +68526,7 @@
     <row r="748">
       <c r="A748" t="inlineStr">
         <is>
-          <t>Atualizado: 03/10/2026 11:29 | Total dias: 745</t>
+          <t>Atualizado: 04/10/2026 12:03 | Total dias: 745</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-05 19:00 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G118"/>
+  <dimension ref="A1:G119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4812,6 +4812,43 @@
         </is>
       </c>
       <c r="G118" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>05/10/2026 15:58</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>6636</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>187</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -11529,7 +11566,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>145</t>
+          <t>146</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -11637,7 +11674,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>223</t>
+          <t>224</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -32763,7 +32800,7 @@
       </c>
       <c r="F534" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G534" t="inlineStr">
@@ -39727,7 +39764,7 @@
     <row r="669">
       <c r="A669" t="inlineStr">
         <is>
-          <t>Atualizado: 04/10/2026 12:03 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 05/10/2026 15:58 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -58798,7 +58835,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 04/10/2026 12:03 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 05/10/2026 15:58 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -58813,7 +58850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C748"/>
+  <dimension ref="A1:C749"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68523,10 +68560,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="748">
-      <c r="A748" t="inlineStr">
-        <is>
-          <t>Atualizado: 04/10/2026 12:03 | Total dias: 745</t>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>05/10/2026</t>
+        </is>
+      </c>
+      <c r="B747" t="n">
+        <v>3</v>
+      </c>
+      <c r="C747" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>Atualizado: 05/10/2026 15:58 | Total dias: 746</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-06 16:24 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G119"/>
+  <dimension ref="A1:G120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4849,6 +4849,43 @@
         </is>
       </c>
       <c r="G119" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>06/10/2026 13:22</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>6644</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>187</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -11935,7 +11972,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -14347,7 +14384,7 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
@@ -26689,7 +26726,7 @@
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>66</t>
         </is>
       </c>
       <c r="G417" t="inlineStr">
@@ -34626,7 +34663,7 @@
       </c>
       <c r="F569" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G569" t="inlineStr">
@@ -34782,7 +34819,7 @@
       </c>
       <c r="F572" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G572" t="inlineStr">
@@ -37703,7 +37740,7 @@
       </c>
       <c r="F628" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G628" t="inlineStr">
@@ -39764,7 +39801,7 @@
     <row r="669">
       <c r="A669" t="inlineStr">
         <is>
-          <t>Atualizado: 05/10/2026 15:58 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 06/10/2026 13:22 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -58835,7 +58872,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 05/10/2026 15:58 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 06/10/2026 13:22 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -58850,7 +58887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C749"/>
+  <dimension ref="A1:C750"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68567,16 +68604,29 @@
         </is>
       </c>
       <c r="B747" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C747" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="749">
-      <c r="A749" t="inlineStr">
-        <is>
-          <t>Atualizado: 05/10/2026 15:58 | Total dias: 746</t>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="B748" t="n">
+        <v>4</v>
+      </c>
+      <c r="C748" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>Atualizado: 06/10/2026 13:22 | Total dias: 747</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-07 17:10 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G120"/>
+  <dimension ref="A1:G121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4886,6 +4886,43 @@
         </is>
       </c>
       <c r="G120" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>07/10/2026 14:07</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>6648</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>187</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -8710,7 +8747,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>381</t>
+          <t>382</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -11711,7 +11748,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>224</t>
+          <t>225</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -29491,7 +29528,7 @@
       </c>
       <c r="F470" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G470" t="inlineStr">
@@ -37792,7 +37829,7 @@
       </c>
       <c r="F629" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>237</t>
         </is>
       </c>
       <c r="G629" t="inlineStr">
@@ -39801,7 +39838,7 @@
     <row r="669">
       <c r="A669" t="inlineStr">
         <is>
-          <t>Atualizado: 06/10/2026 13:22 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 07/10/2026 14:07 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -58872,7 +58909,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 06/10/2026 13:22 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 07/10/2026 14:07 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -58887,7 +58924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C750"/>
+  <dimension ref="A1:C751"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68617,16 +68654,29 @@
         </is>
       </c>
       <c r="B748" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C748" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="750">
-      <c r="A750" t="inlineStr">
-        <is>
-          <t>Atualizado: 06/10/2026 13:22 | Total dias: 747</t>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="B749" t="n">
+        <v>1</v>
+      </c>
+      <c r="C749" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>Atualizado: 07/10/2026 14:07 | Total dias: 748</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-09 16:45 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G122"/>
+  <dimension ref="A1:G123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4960,6 +4960,43 @@
         </is>
       </c>
       <c r="G122" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>09/10/2026 13:43</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>6665</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -9895,7 +9932,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -23975,7 +24012,7 @@
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>75</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
@@ -37655,7 +37692,7 @@
       </c>
       <c r="F625" t="inlineStr">
         <is>
-          <t>237</t>
+          <t>239</t>
         </is>
       </c>
       <c r="G625" t="inlineStr">
@@ -39664,7 +39701,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 08/10/2026 14:06 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 09/10/2026 13:43 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -58735,7 +58772,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 08/10/2026 14:06 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 09/10/2026 13:43 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -58750,7 +58787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C752"/>
+  <dimension ref="A1:C753"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68506,16 +68543,29 @@
         </is>
       </c>
       <c r="B750" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C750" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="752">
-      <c r="A752" t="inlineStr">
-        <is>
-          <t>Atualizado: 08/10/2026 14:06 | Total dias: 749</t>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="B751" t="n">
+        <v>6</v>
+      </c>
+      <c r="C751" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>Atualizado: 09/10/2026 13:43 | Total dias: 750</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-10 15:43 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G123"/>
+  <dimension ref="A1:G124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -4997,6 +4997,43 @@
         </is>
       </c>
       <c r="G123" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>10/10/2026 12:41</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>6669</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -10981,7 +11018,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>147</t>
+          <t>148</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -31377,7 +31414,7 @@
       </c>
       <c r="F504" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="G504" t="inlineStr">
@@ -31691,7 +31728,7 @@
       </c>
       <c r="F510" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>145</t>
         </is>
       </c>
       <c r="G510" t="inlineStr">
@@ -37692,7 +37729,7 @@
       </c>
       <c r="F625" t="inlineStr">
         <is>
-          <t>239</t>
+          <t>240</t>
         </is>
       </c>
       <c r="G625" t="inlineStr">
@@ -39701,7 +39738,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 09/10/2026 13:43 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 10/10/2026 12:41 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -58772,7 +58809,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 09/10/2026 13:43 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 10/10/2026 12:41 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -58787,7 +58824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C753"/>
+  <dimension ref="A1:C754"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68562,10 +68599,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="753">
-      <c r="A753" t="inlineStr">
-        <is>
-          <t>Atualizado: 09/10/2026 13:43 | Total dias: 750</t>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="B752" t="n">
+        <v>4</v>
+      </c>
+      <c r="C752" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>Atualizado: 10/10/2026 12:41 | Total dias: 751</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-11 16:05 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G124"/>
+  <dimension ref="A1:G125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -5034,6 +5034,43 @@
         </is>
       </c>
       <c r="G124" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>11/10/2026 13:03</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>6670</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -10178,7 +10215,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -39738,7 +39775,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 10/10/2026 12:41 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 11/10/2026 13:03 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -58809,7 +58846,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 10/10/2026 12:41 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 11/10/2026 13:03 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -58824,7 +58861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C754"/>
+  <dimension ref="A1:C755"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68612,10 +68649,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="754">
-      <c r="A754" t="inlineStr">
-        <is>
-          <t>Atualizado: 10/10/2026 12:41 | Total dias: 751</t>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>11/10/2026</t>
+        </is>
+      </c>
+      <c r="B753" t="n">
+        <v>1</v>
+      </c>
+      <c r="C753" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>Atualizado: 11/10/2026 13:03 | Total dias: 752</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-12 19:34 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G125"/>
+  <dimension ref="A1:G126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -5071,6 +5071,43 @@
         </is>
       </c>
       <c r="G125" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>12/10/2026 16:32</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>6672</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -31765,7 +31802,7 @@
       </c>
       <c r="F510" t="inlineStr">
         <is>
-          <t>145</t>
+          <t>146</t>
         </is>
       </c>
       <c r="G510" t="inlineStr">
@@ -33177,7 +33214,7 @@
       </c>
       <c r="F537" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="G537" t="inlineStr">
@@ -39775,7 +39812,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 11/10/2026 13:03 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 12/10/2026 16:32 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -58846,7 +58883,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 11/10/2026 13:03 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 12/10/2026 16:32 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -58861,7 +58898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C755"/>
+  <dimension ref="A1:C756"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68656,16 +68693,29 @@
         </is>
       </c>
       <c r="B753" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C753" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="755">
-      <c r="A755" t="inlineStr">
-        <is>
-          <t>Atualizado: 11/10/2026 13:03 | Total dias: 752</t>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="B754" t="n">
+        <v>1</v>
+      </c>
+      <c r="C754" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>Atualizado: 12/10/2026 16:32 | Total dias: 753</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-13 17:17 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G126"/>
+  <dimension ref="A1:G127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -5108,6 +5108,43 @@
         </is>
       </c>
       <c r="G126" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>13/10/2026 14:15</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>6679</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -7105,7 +7142,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -7835,7 +7872,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -12194,7 +12231,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -20676,7 +20713,7 @@
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G297" t="inlineStr">
@@ -28826,7 +28863,7 @@
       </c>
       <c r="F453" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="G453" t="inlineStr">
@@ -31802,7 +31839,7 @@
       </c>
       <c r="F510" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>147</t>
         </is>
       </c>
       <c r="G510" t="inlineStr">
@@ -37281,7 +37318,7 @@
       </c>
       <c r="F615" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G615" t="inlineStr">
@@ -39812,7 +39849,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 12/10/2026 16:32 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 13/10/2026 14:15 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -58883,7 +58920,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 12/10/2026 16:32 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 13/10/2026 14:15 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -58898,7 +58935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C756"/>
+  <dimension ref="A1:C757"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68712,10 +68749,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="756">
-      <c r="A756" t="inlineStr">
-        <is>
-          <t>Atualizado: 12/10/2026 16:32 | Total dias: 753</t>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
+      <c r="B755" t="n">
+        <v>7</v>
+      </c>
+      <c r="C755" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>Atualizado: 13/10/2026 14:15 | Total dias: 754</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-14 14:50 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G127"/>
+  <dimension ref="A1:G128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -5145,6 +5145,43 @@
         </is>
       </c>
       <c r="G127" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>14/10/2026 11:48</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>6682</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -6098,7 +6135,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -13963,7 +14000,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
@@ -37578,7 +37615,7 @@
       </c>
       <c r="F620" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G620" t="inlineStr">
@@ -39849,7 +39886,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 13/10/2026 14:15 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 14/10/2026 11:48 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -58920,7 +58957,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 13/10/2026 14:15 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 14/10/2026 11:48 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -58935,7 +58972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C757"/>
+  <dimension ref="A1:C758"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68756,16 +68793,29 @@
         </is>
       </c>
       <c r="B755" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C755" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="757">
-      <c r="A757" t="inlineStr">
-        <is>
-          <t>Atualizado: 13/10/2026 14:15 | Total dias: 754</t>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>14/10/2026</t>
+        </is>
+      </c>
+      <c r="B756" t="n">
+        <v>1</v>
+      </c>
+      <c r="C756" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>Atualizado: 14/10/2026 11:48 | Total dias: 755</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-15 14:35 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G128"/>
+  <dimension ref="A1:G129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -5182,6 +5182,43 @@
         </is>
       </c>
       <c r="G128" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>15/10/2026 11:32</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>6688</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -5293,7 +5330,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -10379,7 +10416,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -11899,7 +11936,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>147</t>
+          <t>148</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -12687,7 +12724,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
@@ -39886,7 +39923,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 14/10/2026 11:48 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 15/10/2026 11:32 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -58957,7 +58994,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 14/10/2026 11:48 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 15/10/2026 11:32 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -58972,7 +59009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C758"/>
+  <dimension ref="A1:C759"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68806,16 +68843,29 @@
         </is>
       </c>
       <c r="B756" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C756" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="758">
-      <c r="A758" t="inlineStr">
-        <is>
-          <t>Atualizado: 14/10/2026 11:48 | Total dias: 755</t>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="B757" t="n">
+        <v>4</v>
+      </c>
+      <c r="C757" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>Atualizado: 15/10/2026 11:32 | Total dias: 756</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-16 14:26 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G129"/>
+  <dimension ref="A1:G130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -5219,6 +5219,43 @@
         </is>
       </c>
       <c r="G129" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>16/10/2026 11:24</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>6691</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -13985,7 +14022,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>154</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -35254,7 +35291,7 @@
       </c>
       <c r="F574" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G574" t="inlineStr">
@@ -37131,7 +37168,7 @@
       </c>
       <c r="F610" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G610" t="inlineStr">
@@ -39923,7 +39960,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 15/10/2026 11:32 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 16/10/2026 11:24 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -58994,7 +59031,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 15/10/2026 11:32 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 16/10/2026 11:24 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -68856,7 +68893,7 @@
         </is>
       </c>
       <c r="B757" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C757" t="n">
         <v>0</v>
@@ -68865,7 +68902,7 @@
     <row r="759">
       <c r="A759" t="inlineStr">
         <is>
-          <t>Atualizado: 15/10/2026 11:32 | Total dias: 756</t>
+          <t>Atualizado: 16/10/2026 11:24 | Total dias: 756</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-17 13:25 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G130"/>
+  <dimension ref="A1:G131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -5256,6 +5256,43 @@
         </is>
       </c>
       <c r="G130" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>17/10/2026 10:22</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>6693</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -24533,7 +24570,7 @@
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G368" t="inlineStr">
@@ -32524,7 +32561,7 @@
       </c>
       <c r="F521" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="G521" t="inlineStr">
@@ -39960,7 +39997,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 16/10/2026 11:24 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 17/10/2026 10:22 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -59031,7 +59068,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 16/10/2026 11:24 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 17/10/2026 10:22 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -59046,7 +59083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C759"/>
+  <dimension ref="A1:C760"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68899,10 +68936,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="759">
-      <c r="A759" t="inlineStr">
-        <is>
-          <t>Atualizado: 16/10/2026 11:24 | Total dias: 756</t>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="B758" t="n">
+        <v>2</v>
+      </c>
+      <c r="C758" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>Atualizado: 17/10/2026 10:22 | Total dias: 757</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-18 13:44 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G131"/>
+  <dimension ref="A1:G132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -5293,6 +5293,43 @@
         </is>
       </c>
       <c r="G131" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>18/10/2026 10:42</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>6694</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -14007,7 +14044,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>99</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
@@ -39997,7 +40034,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 17/10/2026 10:22 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 18/10/2026 10:42 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -59068,7 +59105,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 17/10/2026 10:22 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 18/10/2026 10:42 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -68943,7 +68980,7 @@
         </is>
       </c>
       <c r="B758" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C758" t="n">
         <v>0</v>
@@ -68952,7 +68989,7 @@
     <row r="760">
       <c r="A760" t="inlineStr">
         <is>
-          <t>Atualizado: 17/10/2026 10:22 | Total dias: 757</t>
+          <t>Atualizado: 18/10/2026 10:42 | Total dias: 757</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-19 16:47 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G132"/>
+  <dimension ref="A1:G133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -5330,6 +5330,43 @@
         </is>
       </c>
       <c r="G132" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>19/10/2026 13:44</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>6697</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -27117,7 +27154,7 @@
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>67</t>
         </is>
       </c>
       <c r="G416" t="inlineStr">
@@ -32024,7 +32061,7 @@
       </c>
       <c r="F510" t="inlineStr">
         <is>
-          <t>147</t>
+          <t>148</t>
         </is>
       </c>
       <c r="G510" t="inlineStr">
@@ -40034,7 +40071,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 18/10/2026 10:42 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 19/10/2026 13:44 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -59105,7 +59142,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 18/10/2026 10:42 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 19/10/2026 13:44 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -59120,7 +59157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C760"/>
+  <dimension ref="A1:C761"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -68986,10 +69023,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="760">
-      <c r="A760" t="inlineStr">
-        <is>
-          <t>Atualizado: 18/10/2026 10:42 | Total dias: 757</t>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="B759" t="n">
+        <v>3</v>
+      </c>
+      <c r="C759" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>Atualizado: 19/10/2026 13:44 | Total dias: 758</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-21 14:50 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G133"/>
+  <dimension ref="A1:G134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -5367,6 +5367,43 @@
         </is>
       </c>
       <c r="G133" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>21/10/2026 11:47</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>6701</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -7989,7 +8026,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>70</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -25380,7 +25417,7 @@
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>86</t>
         </is>
       </c>
       <c r="G382" t="inlineStr">
@@ -40071,7 +40108,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 19/10/2026 13:44 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 21/10/2026 11:47 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -59142,7 +59179,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 19/10/2026 13:44 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 21/10/2026 11:47 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -59157,7 +59194,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C761"/>
+  <dimension ref="A1:C763"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -69036,10 +69073,36 @@
         <v>0</v>
       </c>
     </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="B760" t="n">
+        <v>3</v>
+      </c>
+      <c r="C760" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="761">
       <c r="A761" t="inlineStr">
         <is>
-          <t>Atualizado: 19/10/2026 13:44 | Total dias: 758</t>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="B761" t="n">
+        <v>1</v>
+      </c>
+      <c r="C761" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>Atualizado: 21/10/2026 11:47 | Total dias: 760</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-22 14:49 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G134"/>
+  <dimension ref="A1:G135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -5404,6 +5404,43 @@
         </is>
       </c>
       <c r="G134" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>22/10/2026 11:46</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>6706</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -12229,7 +12266,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>226</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -32045,7 +32082,7 @@
       </c>
       <c r="F509" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="G509" t="inlineStr">
@@ -36223,7 +36260,7 @@
       </c>
       <c r="F589" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G589" t="inlineStr">
@@ -40108,7 +40145,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 21/10/2026 11:47 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 22/10/2026 11:46 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -59179,7 +59216,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 21/10/2026 11:47 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 22/10/2026 11:46 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -59194,7 +59231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C763"/>
+  <dimension ref="A1:C764"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -69093,16 +69130,29 @@
         </is>
       </c>
       <c r="B761" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C761" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="763">
-      <c r="A763" t="inlineStr">
-        <is>
-          <t>Atualizado: 21/10/2026 11:47 | Total dias: 760</t>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="B762" t="n">
+        <v>3</v>
+      </c>
+      <c r="C762" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>Atualizado: 22/10/2026 11:46 | Total dias: 761</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-23 14:35 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G135"/>
+  <dimension ref="A1:G136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -5441,6 +5441,43 @@
         </is>
       </c>
       <c r="G135" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>23/10/2026 11:33</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>6708</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -8845,7 +8882,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -12266,7 +12303,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>227</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -40145,7 +40182,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 22/10/2026 11:46 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 23/10/2026 11:33 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -59216,7 +59253,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 22/10/2026 11:46 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 23/10/2026 11:33 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -59231,7 +59268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C764"/>
+  <dimension ref="A1:C765"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -69149,10 +69186,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="764">
-      <c r="A764" t="inlineStr">
-        <is>
-          <t>Atualizado: 22/10/2026 11:46 | Total dias: 761</t>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
+      <c r="B763" t="n">
+        <v>2</v>
+      </c>
+      <c r="C763" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>Atualizado: 23/10/2026 11:33 | Total dias: 762</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-24 13:45 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G136"/>
+  <dimension ref="A1:G137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -5478,6 +5478,43 @@
         </is>
       </c>
       <c r="G136" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>24/10/2026 10:42</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>6712</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -14244,7 +14281,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>154</t>
+          <t>155</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -30555,7 +30592,7 @@
       </c>
       <c r="F479" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G479" t="inlineStr">
@@ -40182,7 +40219,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 23/10/2026 11:33 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 24/10/2026 10:42 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -59253,7 +59290,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 23/10/2026 11:33 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 24/10/2026 10:42 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -59268,7 +59305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C765"/>
+  <dimension ref="A1:C766"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -69193,16 +69230,29 @@
         </is>
       </c>
       <c r="B763" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C763" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="765">
-      <c r="A765" t="inlineStr">
-        <is>
-          <t>Atualizado: 23/10/2026 11:33 | Total dias: 762</t>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>24/10/2026</t>
+        </is>
+      </c>
+      <c r="B764" t="n">
+        <v>1</v>
+      </c>
+      <c r="C764" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>Atualizado: 24/10/2026 10:42 | Total dias: 763</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-25 14:03 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G137"/>
+  <dimension ref="A1:G138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -5515,6 +5515,43 @@
         </is>
       </c>
       <c r="G137" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>25/10/2026 11:01</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>6714</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -40219,7 +40256,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 24/10/2026 10:42 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 25/10/2026 11:01 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -59290,7 +59327,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 24/10/2026 10:42 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 25/10/2026 11:01 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -69243,7 +69280,7 @@
         </is>
       </c>
       <c r="B764" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C764" t="n">
         <v>0</v>
@@ -69252,7 +69289,7 @@
     <row r="766">
       <c r="A766" t="inlineStr">
         <is>
-          <t>Atualizado: 24/10/2026 10:42 | Total dias: 763</t>
+          <t>Atualizado: 25/10/2026 11:01 | Total dias: 763</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-26 16:26 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G138"/>
+  <dimension ref="A1:G139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -5552,6 +5552,43 @@
         </is>
       </c>
       <c r="G138" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>26/10/2026 13:23</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>6717</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -12269,7 +12306,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>149</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -19452,7 +19489,7 @@
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G265" t="inlineStr">
@@ -39760,7 +39797,7 @@
       </c>
       <c r="F654" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G654" t="inlineStr">
@@ -40256,7 +40293,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 25/10/2026 11:01 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 26/10/2026 13:23 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -59327,7 +59364,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 25/10/2026 11:01 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 26/10/2026 13:23 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -59342,7 +59379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C766"/>
+  <dimension ref="A1:C767"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -69286,10 +69323,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="766">
-      <c r="A766" t="inlineStr">
-        <is>
-          <t>Atualizado: 25/10/2026 11:01 | Total dias: 763</t>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="B765" t="n">
+        <v>3</v>
+      </c>
+      <c r="C765" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>Atualizado: 26/10/2026 13:23 | Total dias: 764</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-28 16:23 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G139"/>
+  <dimension ref="A1:G140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -5589,6 +5589,43 @@
         </is>
       </c>
       <c r="G139" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>28/10/2026 13:21</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>6728</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -6436,7 +6473,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -9627,7 +9664,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -23720,7 +23757,7 @@
       </c>
       <c r="F346" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
@@ -32283,7 +32320,7 @@
       </c>
       <c r="F510" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>149</t>
         </is>
       </c>
       <c r="G510" t="inlineStr">
@@ -40293,7 +40330,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 26/10/2026 13:23 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 28/10/2026 13:21 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -59364,7 +59401,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 26/10/2026 13:23 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 28/10/2026 13:21 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -59379,7 +59416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C767"/>
+  <dimension ref="A1:C770"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -69336,10 +69373,49 @@
         <v>0</v>
       </c>
     </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>26/10/2026</t>
+        </is>
+      </c>
+      <c r="B766" t="n">
+        <v>1</v>
+      </c>
+      <c r="C766" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="767">
       <c r="A767" t="inlineStr">
         <is>
-          <t>Atualizado: 26/10/2026 13:23 | Total dias: 764</t>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="B767" t="n">
+        <v>5</v>
+      </c>
+      <c r="C767" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="B768" t="n">
+        <v>5</v>
+      </c>
+      <c r="C768" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>Atualizado: 28/10/2026 13:21 | Total dias: 767</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-29 16:35 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G140"/>
+  <dimension ref="A1:G141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -5626,6 +5626,43 @@
         </is>
       </c>
       <c r="G140" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>29/10/2026 13:32</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>6729</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -40330,7 +40367,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 28/10/2026 13:21 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 29/10/2026 13:32 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -59401,7 +59438,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 28/10/2026 13:21 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 29/10/2026 13:32 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -69406,7 +69443,7 @@
         </is>
       </c>
       <c r="B768" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C768" t="n">
         <v>0</v>
@@ -69415,7 +69452,7 @@
     <row r="770">
       <c r="A770" t="inlineStr">
         <is>
-          <t>Atualizado: 28/10/2026 13:21 | Total dias: 767</t>
+          <t>Atualizado: 29/10/2026 13:32 | Total dias: 767</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-30 16:27 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G141"/>
+  <dimension ref="A1:G142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -5663,6 +5663,43 @@
         </is>
       </c>
       <c r="G141" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>30/10/2026 13:23</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>6734</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -8233,7 +8270,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>144</t>
+          <t>145</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -40367,7 +40404,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 29/10/2026 13:32 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 30/10/2026 13:23 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -59438,7 +59475,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 29/10/2026 13:32 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 30/10/2026 13:23 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -59453,7 +59490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C770"/>
+  <dimension ref="A1:C772"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -69449,10 +69486,36 @@
         <v>0</v>
       </c>
     </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>29/10/2026</t>
+        </is>
+      </c>
+      <c r="B769" t="n">
+        <v>2</v>
+      </c>
+      <c r="C769" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="770">
       <c r="A770" t="inlineStr">
         <is>
-          <t>Atualizado: 29/10/2026 13:32 | Total dias: 767</t>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="B770" t="n">
+        <v>3</v>
+      </c>
+      <c r="C770" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>Atualizado: 30/10/2026 13:23 | Total dias: 769</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard: 2026-10-31 15:39 UTC
</commit_message>
<xml_diff>
--- a/greenlife_scraper/dados_greenlife.xlsx
+++ b/greenlife_scraper/dados_greenlife.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G142"/>
+  <dimension ref="A1:G143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="2"/>
@@ -5700,6 +5700,43 @@
         </is>
       </c>
       <c r="G142" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>31/10/2026 12:35</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>6737</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
         <is>
           <t>515</t>
         </is>
@@ -29783,7 +29820,7 @@
       </c>
       <c r="F460" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G460" t="inlineStr">
@@ -40404,7 +40441,7 @@
     <row r="665">
       <c r="A665" t="inlineStr">
         <is>
-          <t>Atualizado: 30/10/2026 13:23 | Ativas: 850 | Inativas: 0</t>
+          <t>Atualizado: 31/10/2026 12:35 | Ativas: 850 | Inativas: 0</t>
         </is>
       </c>
     </row>
@@ -59475,7 +59512,7 @@
     <row r="715">
       <c r="A715" t="inlineStr">
         <is>
-          <t>Atualizado: 30/10/2026 13:23 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
+          <t>Atualizado: 31/10/2026 12:35 | Total: 712 | c/ usuario: 197 | s/ usuario: 515</t>
         </is>
       </c>
     </row>
@@ -59490,7 +59527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C772"/>
+  <dimension ref="A1:C773"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -69506,16 +69543,29 @@
         </is>
       </c>
       <c r="B770" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C770" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="772">
-      <c r="A772" t="inlineStr">
-        <is>
-          <t>Atualizado: 30/10/2026 13:23 | Total dias: 769</t>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="B771" t="n">
+        <v>1</v>
+      </c>
+      <c r="C771" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>Atualizado: 31/10/2026 12:35 | Total dias: 770</t>
         </is>
       </c>
     </row>

</xml_diff>